<commit_message>
Capture Citi import pending classification
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R0901a6acd1684dc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R8470d1e572c547fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R07c1c7162a1f4351"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R430e34ca12fc448b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R9d0a7bd5a2c54ecd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="Rc89d2fd7c70c44a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="Rab3fa422e0604807"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R682b6749c1e74aa1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R0b0227d0e8d84410"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R78bce0ea32a048a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R39d7775e8ee447e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="Ra75c3158ff5345d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R004bbefb42c6411b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R1688b20d837642e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R7071d36d6cc24081"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R09c3fa6f4b4c4f40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R873b463c6a53491d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R463df91be4814ed3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="Rc58348e8b57844a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R6e4eaf15c4744596"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R1c9185d8dff74846"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="Ra2ae86bf73924f01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R3c27b25faa924467"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R581d3dd3b37b4428"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="Rd4b2df70123a4b74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="Rc84446122f04428a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R364e0daba8774aa0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R28443546527e40bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R48e2de062d614af3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R5716a34a60614dce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2304,7 +2304,7 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="30">
+  <x:dxfs count="32">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -2558,6 +2558,17 @@
     <x:dxf>
       <x:font>
         <x:b/>
+        <x:color rgb="FF7C5E10"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
         <x:color rgb="FF167C3B"/>
       </x:font>
       <x:fill>
@@ -2606,6 +2617,17 @@
       <x:fill>
         <x:patternFill patternType="solid">
           <x:bgColor rgb="FFDFF3EF"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF7C5E10"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -3002,7 +3024,7 @@
       <x:c r="D9" s="423"/>
       <x:c r="E9" s="405" t="str">
         <x:f>'Support - Account Snapshots'!I16</x:f>
-        <x:v>Needed</x:v>
+        <x:v>Needs classification</x:v>
       </x:c>
       <x:c r="F9" s="406" t="str">
         <x:v>Citi AAdvantage</x:v>
@@ -3118,7 +3140,7 @@
       </x:c>
       <x:c r="B14" s="415" t="n">
         <x:f>COUNTBLANK('Support - Debt Detail'!D5:D15)</x:f>
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C14" s="407" t="str">
         <x:v>Update yellow due-date cells when the account screen or statement shows them</x:v>
@@ -3160,7 +3182,7 @@
       </x:c>
       <x:c r="B16" s="415" t="n">
         <x:f>COUNTIF('Support - Ledger'!E5:E304,"Pending")</x:f>
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C16" s="407" t="str">
         <x:v>Capture every pending item and keep unclear amounts flagged</x:v>
@@ -3201,16 +3223,17 @@
     <x:mergeCell ref="E16:H17"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="B12:B16">
-    <x:cfRule type="cellIs" dxfId="26" priority="1" operator="greaterThan">
+    <x:cfRule type="cellIs" dxfId="27" priority="1" operator="greaterThan">
       <x:formula>0</x:formula>
     </x:cfRule>
-    <x:cfRule type="cellIs" dxfId="27" priority="2" operator="equal">
+    <x:cfRule type="cellIs" dxfId="28" priority="2" operator="equal">
       <x:formula>0</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="E6:E13">
-    <x:cfRule type="containsText" dxfId="28" priority="3" operator="containsText" text="Needed"/>
-    <x:cfRule type="containsText" dxfId="29" priority="4" operator="containsText" text="Source check"/>
+    <x:cfRule type="containsText" dxfId="29" priority="3" operator="containsText" text="Needs classification"/>
+    <x:cfRule type="containsText" dxfId="30" priority="4" operator="containsText" text="Needed"/>
+    <x:cfRule type="containsText" dxfId="31" priority="5" operator="containsText" text="Source check"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3312,12 +3335,14 @@
         <x:v>Citi card</x:v>
       </x:c>
       <x:c r="B6" s="547" t="n">
-        <x:v>132.09</x:v>
+        <x:v>106.26</x:v>
       </x:c>
       <x:c r="C6" s="547" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D6" s="479"/>
+      <x:c r="D6" s="479" t="n">
+        <x:v>46298</x:v>
+      </x:c>
       <x:c r="E6" s="423" t="str">
         <x:v>APR not rechecked</x:v>
       </x:c>
@@ -3325,7 +3350,7 @@
         <x:v>USD</x:v>
       </x:c>
       <x:c r="G6" s="423" t="str">
-        <x:v>Current balance from Sep. 9 Citi screenshot. Closing date Oct. 7; payment due date was not shown.</x:v>
+        <x:v>Current balance from Sep. 15 Citi screenshot. Pending $63.79 is tracked separately; app shows $0.00 statement balance and $0.00 minimum payment.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -4082,7 +4107,7 @@
       </x:c>
       <x:c r="H14" s="423" t="str"/>
       <x:c r="I14" s="423" t="str">
-        <x:f>IF(D14="","Needed",IF(E14&lt;&gt;D14,"Missing entry",IF(ABS(G14-F14)&gt;0.005,"Total mismatch",IF(H14&lt;&gt;"Yes","Anchor not reached","Verified"))))</x:f>
+        <x:f>IF(D14="","Needed",IF(COUNTIFS('Support - Ledger'!$K$5:$K$304,B14,'Support - Ledger'!$M$5:$M$304,"Needs verification")&gt;0,"Needs classification",IF(E14&lt;&gt;D14,"Missing entry",IF(ABS(G14-F14)&gt;0.005,"Total mismatch",IF(H14&lt;&gt;"Yes","Anchor not reached","Verified")))))</x:f>
         <x:v>Needed</x:v>
       </x:c>
       <x:c r="J14" s="423" t="str">
@@ -4111,7 +4136,7 @@
       </x:c>
       <x:c r="H15" s="423" t="str"/>
       <x:c r="I15" s="423" t="str">
-        <x:f>IF(D15="","Needed",IF(E15&lt;&gt;D15,"Missing entry",IF(ABS(G15-F15)&gt;0.005,"Total mismatch",IF(H15&lt;&gt;"Yes","Anchor not reached","Verified"))))</x:f>
+        <x:f>IF(D15="","Needed",IF(COUNTIFS('Support - Ledger'!$K$5:$K$304,B15,'Support - Ledger'!$M$5:$M$304,"Needs verification")&gt;0,"Needs classification",IF(E15&lt;&gt;D15,"Missing entry",IF(ABS(G15-F15)&gt;0.005,"Total mismatch",IF(H15&lt;&gt;"Yes","Anchor not reached","Verified")))))</x:f>
         <x:v>Needed</x:v>
       </x:c>
       <x:c r="J15" s="423" t="str">
@@ -4126,25 +4151,31 @@
         <x:v>Citi activity — Sep 15</x:v>
       </x:c>
       <x:c r="C16" s="423" t="str">
-        <x:v>Posted ledger rows</x:v>
-      </x:c>
-      <x:c r="D16" s="423" t="str"/>
+        <x:v>Posted + pending ledger rows</x:v>
+      </x:c>
+      <x:c r="D16" s="423" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="E16" s="423" t="n">
         <x:f>COUNTIF('Support - Ledger'!$K$5:$K$304,B16)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F16" s="481" t="str"/>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F16" s="481" t="n">
+        <x:v>37.96</x:v>
+      </x:c>
       <x:c r="G16" s="481" t="n">
         <x:f>SUMIF('Support - Ledger'!$K$5:$K$304,B16,'Support - Ledger'!$D$5:$D$304)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H16" s="423" t="str"/>
+        <x:v>37.96</x:v>
+      </x:c>
+      <x:c r="H16" s="423" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
       <x:c r="I16" s="423" t="str">
-        <x:f>IF(D16="","Needed",IF(E16&lt;&gt;D16,"Missing entry",IF(ABS(G16-F16)&gt;0.005,"Total mismatch",IF(H16&lt;&gt;"Yes","Anchor not reached","Verified"))))</x:f>
-        <x:v>Needed</x:v>
+        <x:f>IF(D16="","Needed",IF(COUNTIFS('Support - Ledger'!$K$5:$K$304,B16,'Support - Ledger'!$M$5:$M$304,"Needs verification")&gt;0,"Needs classification",IF(E16&lt;&gt;D16,"Missing entry",IF(ABS(G16-F16)&gt;0.005,"Total mismatch",IF(H16&lt;&gt;"Yes","Anchor not reached","Verified")))))</x:f>
+        <x:v>Needs classification</x:v>
       </x:c>
       <x:c r="J16" s="423" t="str">
-        <x:v>Capture posted activity through the saved anchor</x:v>
+        <x:v>Two transactions need category confirmation</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
@@ -4191,7 +4222,7 @@
       </x:c>
       <x:c r="H18" s="423" t="str"/>
       <x:c r="I18" s="423" t="str">
-        <x:f>IF(D18="","Needed",IF(E18&lt;&gt;D18,"Missing entry",IF(ABS(G18-F18)&gt;0.005,"Total mismatch",IF(H18&lt;&gt;"Yes","Anchor not reached","Verified"))))</x:f>
+        <x:f>IF(D18="","Needed",IF(COUNTIFS('Support - Ledger'!$K$5:$K$304,B18,'Support - Ledger'!$M$5:$M$304,"Needs verification")&gt;0,"Needs classification",IF(E18&lt;&gt;D18,"Missing entry",IF(ABS(G18-F18)&gt;0.005,"Total mismatch",IF(H18&lt;&gt;"Yes","Anchor not reached","Verified")))))</x:f>
         <x:v>Needed</x:v>
       </x:c>
       <x:c r="J18" s="423" t="str">
@@ -4274,7 +4305,8 @@
     <x:cfRule type="containsText" dxfId="18" priority="1" operator="containsText" text="Verified"/>
     <x:cfRule type="containsText" dxfId="19" priority="2" operator="containsText" text="Missing"/>
     <x:cfRule type="containsText" dxfId="20" priority="3" operator="containsText" text="mismatch"/>
-    <x:cfRule type="containsText" dxfId="21" priority="4" operator="containsText" text="Needed"/>
+    <x:cfRule type="containsText" dxfId="21" priority="4" operator="containsText" text="Needs classification"/>
+    <x:cfRule type="containsText" dxfId="22" priority="5" operator="containsText" text="Needed"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -5611,7 +5643,6 @@
         <x:v>Current Sep. 9 balance</x:v>
       </x:c>
       <x:c r="D9" s="468" t="n">
-        <x:f>'Support - Debt Detail'!B5</x:f>
         <x:v>266.96</x:v>
       </x:c>
       <x:c r="E9" s="460" t="str">
@@ -5635,7 +5666,6 @@
         <x:v>Current Sep. 9 balance</x:v>
       </x:c>
       <x:c r="D10" s="468" t="n">
-        <x:f>'Support - Debt Detail'!B6</x:f>
         <x:v>132.09</x:v>
       </x:c>
       <x:c r="E10" s="460" t="str">
@@ -5940,10 +5970,10 @@
     <x:mergeCell ref="A24:D24"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="E9:E19">
-    <x:cfRule type="containsText" dxfId="22" priority="1" operator="containsText" text="☐ Pay now"/>
-    <x:cfRule type="containsText" dxfId="23" priority="2" operator="containsText" text="☑ Done"/>
-    <x:cfRule type="containsText" dxfId="24" priority="3" operator="containsText" text="Auto"/>
-    <x:cfRule type="containsText" dxfId="25" priority="4" operator="containsText" text="Not"/>
+    <x:cfRule type="containsText" dxfId="23" priority="1" operator="containsText" text="☐ Pay now"/>
+    <x:cfRule type="containsText" dxfId="24" priority="2" operator="containsText" text="☑ Done"/>
+    <x:cfRule type="containsText" dxfId="25" priority="3" operator="containsText" text="Auto"/>
+    <x:cfRule type="containsText" dxfId="26" priority="4" operator="containsText" text="Not"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="E9:E19">
@@ -8030,7 +8060,7 @@
       <x:c r="H7" s="547"/>
       <x:c r="I7" s="481" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$H$5:$H$304,B7,'Support - Ledger'!$E$5:$E$304,"Posted",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>0</x:v>
+        <x:v>82.79</x:v>
       </x:c>
       <x:c r="J7" s="481" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$H$5:$H$304,B7,'Support - Ledger'!$E$5:$E$304,"Pending",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
@@ -8038,7 +8068,7 @@
       </x:c>
       <x:c r="K7" s="481" t="n">
         <x:f>I7+J7</x:f>
-        <x:v>74.49000000000001</x:v>
+        <x:v>157.28000000000003</x:v>
       </x:c>
       <x:c r="L7" s="481" t="str">
         <x:f>IF(H7="","",H7-K7)</x:f>
@@ -12025,89 +12055,214 @@
       </x:c>
     </x:row>
     <x:row r="78">
-      <x:c r="A78" s="548"/>
-      <x:c r="B78" s="479"/>
-      <x:c r="C78" s="548"/>
-      <x:c r="D78" s="547"/>
-      <x:c r="E78" s="548"/>
-      <x:c r="F78" s="548"/>
-      <x:c r="G78" s="548"/>
-      <x:c r="H78" s="574" t="str">
+      <x:c r="A78" s="548" t="str">
+        <x:v>Citi</x:v>
+      </x:c>
+      <x:c r="B78" s="479" t="n">
+        <x:v>46275</x:v>
+      </x:c>
+      <x:c r="C78" s="548" t="str">
+        <x:v>EXXON CHECKOUT #70 ROCKPORT</x:v>
+      </x:c>
+      <x:c r="D78" s="547" t="n">
+        <x:v>10.01</x:v>
+      </x:c>
+      <x:c r="E78" s="548" t="str">
+        <x:v>Posted</x:v>
+      </x:c>
+      <x:c r="F78" s="548" t="str">
+        <x:v>Fuel</x:v>
+      </x:c>
+      <x:c r="G78" s="548" t="str">
+        <x:v>Include</x:v>
+      </x:c>
+      <x:c r="H78" s="574" t="n">
         <x:f>IF(B78="","",B78-WEEKDAY(B78-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I78" s="548"/>
-      <x:c r="J78" s="548"/>
-      <x:c r="K78" s="548"/>
-      <x:c r="L78" s="548"/>
-      <x:c r="M78" s="548"/>
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="I78" s="548" t="str">
+        <x:v>citi-2026-09-10-exxon-1001</x:v>
+      </x:c>
+      <x:c r="J78" s="548" t="str">
+        <x:v>Fuel purchase visible in Sep. 15 Citi activity</x:v>
+      </x:c>
+      <x:c r="K78" s="548" t="str">
+        <x:v>Citi activity — Sep 15</x:v>
+      </x:c>
+      <x:c r="L78" s="548" t="str">
+        <x:v>Posted activity</x:v>
+      </x:c>
+      <x:c r="M78" s="548" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
     </x:row>
     <x:row r="79">
-      <x:c r="A79" s="548"/>
-      <x:c r="B79" s="479"/>
-      <x:c r="C79" s="548"/>
-      <x:c r="D79" s="547"/>
-      <x:c r="E79" s="548"/>
-      <x:c r="F79" s="548"/>
-      <x:c r="G79" s="548"/>
-      <x:c r="H79" s="574" t="str">
+      <x:c r="A79" s="548" t="str">
+        <x:v>Citi</x:v>
+      </x:c>
+      <x:c r="B79" s="479" t="n">
+        <x:v>46275</x:v>
+      </x:c>
+      <x:c r="C79" s="548" t="str">
+        <x:v>ONLINE PAYMENT, THANK YOU</x:v>
+      </x:c>
+      <x:c r="D79" s="547" t="n">
+        <x:v>-132.09</x:v>
+      </x:c>
+      <x:c r="E79" s="548" t="str">
+        <x:v>Posted</x:v>
+      </x:c>
+      <x:c r="F79" s="548" t="str">
+        <x:v>Credit-card payment</x:v>
+      </x:c>
+      <x:c r="G79" s="548" t="str">
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="H79" s="574" t="n">
         <x:f>IF(B79="","",B79-WEEKDAY(B79-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I79" s="548"/>
-      <x:c r="J79" s="548"/>
-      <x:c r="K79" s="548"/>
-      <x:c r="L79" s="548"/>
-      <x:c r="M79" s="548"/>
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="I79" s="548" t="str">
+        <x:v>citi-2026-09-10-payment-13209</x:v>
+      </x:c>
+      <x:c r="J79" s="548" t="str">
+        <x:v>Card payment confirmed by Citi and Wells; excluded from spending</x:v>
+      </x:c>
+      <x:c r="K79" s="548" t="str">
+        <x:v>Citi activity — Sep 15</x:v>
+      </x:c>
+      <x:c r="L79" s="548" t="str">
+        <x:v>Posted activity</x:v>
+      </x:c>
+      <x:c r="M79" s="548" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
     </x:row>
     <x:row r="80">
-      <x:c r="A80" s="548"/>
-      <x:c r="B80" s="479"/>
-      <x:c r="C80" s="548"/>
-      <x:c r="D80" s="547"/>
-      <x:c r="E80" s="548"/>
-      <x:c r="F80" s="548"/>
-      <x:c r="G80" s="548"/>
-      <x:c r="H80" s="574" t="str">
+      <x:c r="A80" s="548" t="str">
+        <x:v>Citi</x:v>
+      </x:c>
+      <x:c r="B80" s="479" t="n">
+        <x:v>46276</x:v>
+      </x:c>
+      <x:c r="C80" s="548" t="str">
+        <x:v>PCC 9394 INGLESIDE TX</x:v>
+      </x:c>
+      <x:c r="D80" s="547" t="n">
+        <x:v>72.78</x:v>
+      </x:c>
+      <x:c r="E80" s="548" t="str">
+        <x:v>Posted</x:v>
+      </x:c>
+      <x:c r="F80" s="548" t="str">
+        <x:v>Fuel</x:v>
+      </x:c>
+      <x:c r="G80" s="548" t="str">
+        <x:v>Include</x:v>
+      </x:c>
+      <x:c r="H80" s="574" t="n">
         <x:f>IF(B80="","",B80-WEEKDAY(B80-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I80" s="548"/>
-      <x:c r="J80" s="548"/>
-      <x:c r="K80" s="548"/>
-      <x:c r="L80" s="548"/>
-      <x:c r="M80" s="548"/>
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="I80" s="548" t="str">
+        <x:v>citi-2026-09-11-pcc-7278</x:v>
+      </x:c>
+      <x:c r="J80" s="548" t="str">
+        <x:v>Same merchant as the prior verified Citi fuel purchase</x:v>
+      </x:c>
+      <x:c r="K80" s="548" t="str">
+        <x:v>Citi activity — Sep 15</x:v>
+      </x:c>
+      <x:c r="L80" s="548" t="str">
+        <x:v>Posted activity</x:v>
+      </x:c>
+      <x:c r="M80" s="548" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
     </x:row>
     <x:row r="81">
-      <x:c r="A81" s="548"/>
-      <x:c r="B81" s="479"/>
-      <x:c r="C81" s="548"/>
-      <x:c r="D81" s="547"/>
-      <x:c r="E81" s="548"/>
-      <x:c r="F81" s="548"/>
-      <x:c r="G81" s="548"/>
-      <x:c r="H81" s="574" t="str">
+      <x:c r="A81" s="548" t="str">
+        <x:v>Citi</x:v>
+      </x:c>
+      <x:c r="B81" s="479" t="n">
+        <x:v>46277</x:v>
+      </x:c>
+      <x:c r="C81" s="548" t="str">
+        <x:v>WM SUPERCENTER #440 ROCKPORT</x:v>
+      </x:c>
+      <x:c r="D81" s="547" t="n">
+        <x:v>23.47</x:v>
+      </x:c>
+      <x:c r="E81" s="548" t="str">
+        <x:v>Posted</x:v>
+      </x:c>
+      <x:c r="F81" s="548" t="str">
+        <x:v>Unclassified</x:v>
+      </x:c>
+      <x:c r="G81" s="548" t="str">
+        <x:v>Needs classification</x:v>
+      </x:c>
+      <x:c r="H81" s="574" t="n">
         <x:f>IF(B81="","",B81-WEEKDAY(B81-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I81" s="548"/>
-      <x:c r="J81" s="548"/>
-      <x:c r="K81" s="548"/>
-      <x:c r="L81" s="548"/>
-      <x:c r="M81" s="548"/>
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="I81" s="548" t="str">
+        <x:v>citi-2026-09-12-walmart-2347</x:v>
+      </x:c>
+      <x:c r="J81" s="548" t="str">
+        <x:v>Merchant and amount verified; waiting for user category</x:v>
+      </x:c>
+      <x:c r="K81" s="548" t="str">
+        <x:v>Citi activity — Sep 15</x:v>
+      </x:c>
+      <x:c r="L81" s="548" t="str">
+        <x:v>Posted activity</x:v>
+      </x:c>
+      <x:c r="M81" s="548" t="str">
+        <x:v>Needs verification</x:v>
+      </x:c>
     </x:row>
     <x:row r="82">
-      <x:c r="A82" s="548"/>
-      <x:c r="B82" s="479"/>
-      <x:c r="C82" s="548"/>
-      <x:c r="D82" s="547"/>
-      <x:c r="E82" s="548"/>
-      <x:c r="F82" s="548"/>
-      <x:c r="G82" s="548"/>
-      <x:c r="H82" s="574" t="str">
+      <x:c r="A82" s="548" t="str">
+        <x:v>Citi</x:v>
+      </x:c>
+      <x:c r="B82" s="479" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="C82" s="548" t="str">
+        <x:v>SE40845 INGLESIDE USA</x:v>
+      </x:c>
+      <x:c r="D82" s="547" t="n">
+        <x:v>63.79</x:v>
+      </x:c>
+      <x:c r="E82" s="548" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="F82" s="548" t="str">
+        <x:v>Unclassified</x:v>
+      </x:c>
+      <x:c r="G82" s="548" t="str">
+        <x:v>Needs classification</x:v>
+      </x:c>
+      <x:c r="H82" s="574" t="n">
         <x:f>IF(B82="","",B82-WEEKDAY(B82-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I82" s="548"/>
-      <x:c r="J82" s="548"/>
-      <x:c r="K82" s="548"/>
-      <x:c r="L82" s="548"/>
-      <x:c r="M82" s="548"/>
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="I82" s="548" t="str">
+        <x:v>citi-2026-09-14-se40845-6379</x:v>
+      </x:c>
+      <x:c r="J82" s="548" t="str">
+        <x:v>Merchant and amount verified; waiting for user category</x:v>
+      </x:c>
+      <x:c r="K82" s="548" t="str">
+        <x:v>Citi activity — Sep 15</x:v>
+      </x:c>
+      <x:c r="L82" s="548" t="str">
+        <x:v>Pending list</x:v>
+      </x:c>
+      <x:c r="M82" s="548" t="str">
+        <x:v>Needs verification</x:v>
+      </x:c>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="548"/>

</xml_diff>

<commit_message>
Classify current Citi transactions
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R1a8bc604f0644a98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R3da79b4b46c14d05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R693da6cfcee54387"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="Rd32c9bb7eb234e79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R6aba287ef09d4053"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R21169ee496df40d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R1af9154feafe46af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R2ef51c0c80dd49b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="Rf8e52e3e79014468"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R1d7075092faf4f15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R9ba31c3e65de445d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R94e33605aa7441d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="Ra10a67242fa14d15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="Rc90d32f3817c4371"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R21c07e084b5e4dc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R84700ae9219f45a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="Ra588146c60134a98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="Ra99976d544d149a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="Re91fe1e492a845e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R2308a2ed8afa4c9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="Rf6147bb5f1d742cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R07e3d3470ed54ad3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R9efe9cf776454c8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R377bd4e65d8d4608"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R95b62b94c4a54feb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="Rf4e0455b875d4f47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="Ree23d245d72d4275"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R083bd4fe19dd4340"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R97c18eb6a45b449f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="Rd76b54be3bac45b9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3024,7 +3024,7 @@
       <x:c r="D9" s="423"/>
       <x:c r="E9" s="405" t="str">
         <x:f>'Support - Account Snapshots'!I16</x:f>
-        <x:v>Needs classification</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="F9" s="406" t="str">
         <x:v>Citi AAdvantage</x:v>
@@ -4172,7 +4172,7 @@
       </x:c>
       <x:c r="I16" s="423" t="str">
         <x:f>IF(D16="","Needed",IF(COUNTIFS('Support - Ledger'!$K$5:$K$304,B16,'Support - Ledger'!$M$5:$M$304,"Needs verification")&gt;0,"Needs classification",IF(E16&lt;&gt;D16,"Missing entry",IF(ABS(G16-F16)&gt;0.005,"Total mismatch",IF(H16&lt;&gt;"Yes","Anchor not reached","Verified")))))</x:f>
-        <x:v>Needs classification</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="J16" s="423" t="str">
         <x:v>Two transactions need category confirmation</x:v>
@@ -5584,7 +5584,7 @@
     <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="458" t="str">
         <x:f>COUNTIF('1. Start'!E6:E13,"Verified")&amp;" of "&amp;(COUNTA('1. Start'!F6:F14)-COUNTIF('1. Start'!E6:E14,"Not due"))&amp;" source sets verified"</x:f>
-        <x:v>1 of 8 source sets verified</x:v>
+        <x:v>2 of 8 source sets verified</x:v>
       </x:c>
       <x:c r="B6" s="458" t="str">
         <x:v>Sep 1–Sep 7 purchases</x:v>
@@ -8105,15 +8105,15 @@
       <x:c r="H7" s="547"/>
       <x:c r="I7" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$H$5:$H$304,B7,'Support - Ledger'!$E$5:$E$304,"Posted",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>82.79</x:v>
+        <x:v>106.26</x:v>
       </x:c>
       <x:c r="J7" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$H$5:$H$304,B7,'Support - Ledger'!$E$5:$E$304,"Pending",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>74.49000000000001</x:v>
+        <x:v>138.28</x:v>
       </x:c>
       <x:c r="K7" s="480" t="n">
         <x:f>I7+J7</x:f>
-        <x:v>157.28000000000003</x:v>
+        <x:v>244.54000000000002</x:v>
       </x:c>
       <x:c r="L7" s="480" t="str">
         <x:f>IF(H7="","",H7-K7)</x:f>
@@ -12242,10 +12242,10 @@
         <x:v>Posted</x:v>
       </x:c>
       <x:c r="F81" s="548" t="str">
-        <x:v>Unclassified</x:v>
+        <x:v>Car supplies</x:v>
       </x:c>
       <x:c r="G81" s="548" t="str">
-        <x:v>Needs classification</x:v>
+        <x:v>Include</x:v>
       </x:c>
       <x:c r="H81" s="574" t="n">
         <x:f>IF(B81="","",B81-WEEKDAY(B81-2,1)+1)</x:f>
@@ -12255,7 +12255,7 @@
         <x:v>citi-2026-09-12-walmart-2347</x:v>
       </x:c>
       <x:c r="J81" s="548" t="str">
-        <x:v>Merchant and amount verified; waiting for user category</x:v>
+        <x:v>User classified as car supplies</x:v>
       </x:c>
       <x:c r="K81" s="548" t="str">
         <x:v>Citi activity — Sep 15</x:v>
@@ -12264,7 +12264,7 @@
         <x:v>Posted activity</x:v>
       </x:c>
       <x:c r="M81" s="548" t="str">
-        <x:v>Needs verification</x:v>
+        <x:v>Verified</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
@@ -12284,10 +12284,10 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F82" s="548" t="str">
-        <x:v>Unclassified</x:v>
+        <x:v>Fuel</x:v>
       </x:c>
       <x:c r="G82" s="548" t="str">
-        <x:v>Needs classification</x:v>
+        <x:v>Include</x:v>
       </x:c>
       <x:c r="H82" s="574" t="n">
         <x:f>IF(B82="","",B82-WEEKDAY(B82-2,1)+1)</x:f>
@@ -12297,7 +12297,7 @@
         <x:v>citi-2026-09-14-se40845-6379</x:v>
       </x:c>
       <x:c r="J82" s="548" t="str">
-        <x:v>Merchant and amount verified; waiting for user category</x:v>
+        <x:v>User classified as fuel</x:v>
       </x:c>
       <x:c r="K82" s="548" t="str">
         <x:v>Citi activity — Sep 15</x:v>
@@ -12306,7 +12306,7 @@
         <x:v>Pending list</x:v>
       </x:c>
       <x:c r="M82" s="548" t="str">
-        <x:v>Needs verification</x:v>
+        <x:v>Verified</x:v>
       </x:c>
     </x:row>
     <x:row r="83">

</xml_diff>

<commit_message>
Import Chase and account snapshots
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R84700ae9219f45a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="Ra588146c60134a98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="Ra99976d544d149a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="Re91fe1e492a845e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R2308a2ed8afa4c9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="Rf6147bb5f1d742cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R07e3d3470ed54ad3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R9efe9cf776454c8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R377bd4e65d8d4608"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R95b62b94c4a54feb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="Rf4e0455b875d4f47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="Ree23d245d72d4275"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R083bd4fe19dd4340"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R97c18eb6a45b449f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="Rd76b54be3bac45b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R0d58d46c8b0c4216"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R6bdf36e212a84f60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R3d5cdcab761248ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="Rd9b62d36e14a490d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="Rabbfabd2f0114dbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="Rfb86f398aff24cc3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R2b236d01cb8946b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R7b222af8d7e44e89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="Rfd7788d394c74dff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R3fc0106e3fb040b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R3079e3517b414031"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R300128cabed1444a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R5e5c740167cb400b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="Raf532aa1deb34965"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="Rf1bb359141a74d34"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2980,13 +2980,13 @@
       <x:c r="D7" s="423"/>
       <x:c r="E7" s="405" t="str">
         <x:f>'Support - Account Snapshots'!I13</x:f>
-        <x:v>Needed</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="F7" s="406" t="str">
         <x:v>Wealthfront</x:v>
       </x:c>
       <x:c r="G7" s="406" t="str">
-        <x:v>Sep 2 · Wells transfer · $631.34</x:v>
+        <x:v>Sep 14 · Wells Fargo IFI · +$300.00</x:v>
       </x:c>
       <x:c r="H7" s="407" t="str">
         <x:v>Needed</x:v>
@@ -3005,13 +3005,13 @@
       <x:c r="D8" s="423"/>
       <x:c r="E8" s="405" t="str">
         <x:f>IF(AND('Support - Account Snapshots'!I14="Verified",'Support - Account Snapshots'!I15="Verified"),"Verified","Needed")</x:f>
-        <x:v>Needed</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="F8" s="406" t="str">
         <x:v>Chase Sapphire</x:v>
       </x:c>
       <x:c r="G8" s="406" t="str">
-        <x:v>Sep 6 · Card payment · $1,141.57</x:v>
+        <x:v>Sep 13 · Invincible AppCharge · $91.79</x:v>
       </x:c>
       <x:c r="H8" s="407" t="str">
         <x:v>Needed</x:v>
@@ -3096,7 +3096,7 @@
       <x:c r="D12" s="423"/>
       <x:c r="E12" s="405" t="str">
         <x:f>'Support - Account Snapshots'!I19</x:f>
-        <x:v>Needed</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="F12" s="406" t="str">
         <x:v>Capital One</x:v>
@@ -3122,13 +3122,13 @@
       <x:c r="D13" s="423"/>
       <x:c r="E13" s="405" t="str">
         <x:f>'Support - Account Snapshots'!I20</x:f>
-        <x:v>Needed</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="F13" s="406" t="str">
         <x:v>PayPal Credit</x:v>
       </x:c>
       <x:c r="G13" s="406" t="str">
-        <x:v>Sep 2 · payment · $148.65</x:v>
+        <x:v>Sep 10 · payment · $148.62</x:v>
       </x:c>
       <x:c r="H13" s="407" t="str">
         <x:v>Needed</x:v>
@@ -3140,7 +3140,7 @@
       </x:c>
       <x:c r="B14" s="415" t="n">
         <x:f>COUNTBLANK('Support - Debt Detail'!D5:D15)</x:f>
-        <x:v>9</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C14" s="407" t="str">
         <x:v>Update yellow due-date cells when the account screen or statement shows them</x:v>
@@ -3182,7 +3182,7 @@
       </x:c>
       <x:c r="B16" s="415" t="n">
         <x:f>COUNTIF('Support - Ledger'!E5:E304,"Pending")</x:f>
-        <x:v>9</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C16" s="407" t="str">
         <x:v>Capture every pending item and keep unclear amounts flagged</x:v>
@@ -3314,12 +3314,14 @@
         <x:v>Chase card</x:v>
       </x:c>
       <x:c r="B5" s="547" t="n">
-        <x:v>266.96</x:v>
+        <x:v>786.38</x:v>
       </x:c>
       <x:c r="C5" s="547" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D5" s="478"/>
+      <x:c r="D5" s="478" t="n">
+        <x:v>46289</x:v>
+      </x:c>
       <x:c r="E5" s="423" t="str">
         <x:v>27.49% purchases (statement)</x:v>
       </x:c>
@@ -3327,7 +3329,7 @@
         <x:v>USD</x:v>
       </x:c>
       <x:c r="G5" s="423" t="str">
-        <x:v>Current balance from Sep. 9 Chase screenshot. $500.33 pending activity is tracked separately. No payment due was shown.</x:v>
+        <x:v>Current balance from Sep. 15 Chase screenshot. No payment is currently due; $159.54 of current activity is pending and tracked separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -3392,7 +3394,7 @@
         <x:v>USD</x:v>
       </x:c>
       <x:c r="G8" s="423" t="str">
-        <x:v>Current balance $0 in Sep. 9 app screenshot</x:v>
+        <x:v>Current balance $0 in Sep. 15 app screenshot</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -3421,7 +3423,7 @@
         <x:v>PayPal Credit</x:v>
       </x:c>
       <x:c r="B10" s="547" t="n">
-        <x:v>1318.93</x:v>
+        <x:v>1170.31</x:v>
       </x:c>
       <x:c r="C10" s="547" t="n">
         <x:v>0</x:v>
@@ -3434,7 +3436,7 @@
         <x:v>USD</x:v>
       </x:c>
       <x:c r="G10" s="423" t="str">
-        <x:v>Sep. 9 app screenshot; Sep. 2 payment of $148.65 reduced Progressive to $169.37. App warns displayed amounts may be delayed.</x:v>
+        <x:v>Sep. 15 active-promo list totals $1,170.31. The Sep. 10 $148.62 payment reduced Progressive to $20.75.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -3592,7 +3594,7 @@
         <x:v>Reference date</x:v>
       </x:c>
       <x:c r="B3" s="597" t="n">
-        <x:v>46274</x:v>
+        <x:v>46280</x:v>
       </x:c>
       <x:c r="C3" s="573"/>
       <x:c r="D3" s="573" t="str">
@@ -3644,18 +3646,18 @@
         <x:v>46305</x:v>
       </x:c>
       <x:c r="C6" s="599" t="n">
-        <x:v>169.37</x:v>
+        <x:v>20.75</x:v>
       </x:c>
       <x:c r="D6" s="599" t="n">
         <x:v>105.51</x:v>
       </x:c>
       <x:c r="E6" s="573" t="n">
         <x:f>MAX(1,ROUNDUP((B6-$B$3)/7,0))</x:f>
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F6" s="599" t="n">
         <x:f>IF($B$3&gt;B6,0,IF(B6&lt;=$E$3,C6/E6,IF($B$3&gt;$E$3,C6/E6,0)))</x:f>
-        <x:v>33.874</x:v>
+        <x:v>5.1875</x:v>
       </x:c>
       <x:c r="G6" s="573" t="str">
         <x:f>IF(B6&lt;=$E$3,"Stage 1 - pay now",IF($B$3&lt;=$E$3,"Stage 2 - begins after Oct. 10","Stage 2 - pay now"))</x:f>
@@ -3677,11 +3679,11 @@
       </x:c>
       <x:c r="E7" s="573" t="n">
         <x:f>MAX(1,ROUNDUP((B7-$B$3)/7,0))</x:f>
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F7" s="599" t="n">
         <x:f>IF($B$3&gt;B7,0,IF(B7&lt;=$E$3,C7/E7,IF($B$3&gt;$E$3,C7/E7,0)))</x:f>
-        <x:v>114.742</x:v>
+        <x:v>143.4275</x:v>
       </x:c>
       <x:c r="G7" s="573" t="str">
         <x:f>IF(B7&lt;=$E$3,"Stage 1 - pay now",IF($B$3&lt;=$E$3,"Stage 2 - begins after Oct. 10","Stage 2 - pay now"))</x:f>
@@ -3703,7 +3705,7 @@
       </x:c>
       <x:c r="E8" s="573" t="n">
         <x:f>MAX(1,ROUNDUP((B8-$B$3)/7,0))</x:f>
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="F8" s="599" t="n">
         <x:f>IF($B$3&gt;B8,0,IF(B8&lt;=$E$3,C8/E8,IF($B$3&gt;$E$3,C8/E8,0)))</x:f>
@@ -3729,7 +3731,7 @@
       </x:c>
       <x:c r="E9" s="573" t="n">
         <x:f>MAX(1,ROUNDUP((B9-$B$3)/7,0))</x:f>
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="F9" s="599" t="n">
         <x:f>IF($B$3&gt;B9,0,IF(B9&lt;=$E$3,C9/E9,IF($B$3&gt;$E$3,C9/E9,0)))</x:f>
@@ -3756,7 +3758,7 @@
       <x:c r="B11" s="600"/>
       <x:c r="C11" s="601" t="n">
         <x:f>SUM(C6:C9)</x:f>
-        <x:v>1318.93</x:v>
+        <x:v>1170.31</x:v>
       </x:c>
       <x:c r="D11" s="601" t="n">
         <x:f>SUM(D6:D9)</x:f>
@@ -3765,7 +3767,7 @@
       <x:c r="E11" s="600"/>
       <x:c r="F11" s="601" t="n">
         <x:f>SUM(F6:F9)</x:f>
-        <x:v>148.616</x:v>
+        <x:v>148.615</x:v>
       </x:c>
       <x:c r="G11" s="600"/>
     </x:row>
@@ -3779,7 +3781,7 @@
       <x:c r="E12" s="603"/>
       <x:c r="F12" s="604" t="n">
         <x:f>F11</x:f>
-        <x:v>148.616</x:v>
+        <x:v>148.615</x:v>
       </x:c>
       <x:c r="G12" s="605"/>
     </x:row>
@@ -3908,13 +3910,13 @@
     </x:row>
     <x:row r="6" ht="45" customHeight="1">
       <x:c r="A6" s="479" t="n">
-        <x:v>46274</x:v>
+        <x:v>46280</x:v>
       </x:c>
       <x:c r="B6" s="423" t="str">
         <x:v>Wealthfront savings</x:v>
       </x:c>
       <x:c r="C6" s="480" t="n">
-        <x:v>11847.64</x:v>
+        <x:v>12026.13</x:v>
       </x:c>
       <x:c r="D6" s="480" t="n">
         <x:v>0</x:v>
@@ -3923,10 +3925,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F6" s="480" t="n">
-        <x:v>11847.64</x:v>
+        <x:v>12026.13</x:v>
       </x:c>
       <x:c r="G6" s="423" t="str">
-        <x:v>Sep. 9 screenshot; no activity after the Sep. 2 Wells transfer is visible</x:v>
+        <x:v>Sep. 15 balance and activity captured; latest visible activity is the Sep. 14 $300 Wells Fargo IFI transfer.</x:v>
       </x:c>
       <x:c r="H6" s="573"/>
       <x:c r="I6" s="573"/>
@@ -4079,10 +4081,10 @@
       <x:c r="G13" s="480" t="str"/>
       <x:c r="H13" s="423" t="str"/>
       <x:c r="I13" s="423" t="str">
-        <x:v>Needed</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="J13" s="423" t="str">
-        <x:v>Capture the new balance and activity if it changed</x:v>
+        <x:v>Balance and latest activity captured</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="30" customHeight="1">
@@ -4095,23 +4097,29 @@
       <x:c r="C14" s="423" t="str">
         <x:v>Posted ledger rows</x:v>
       </x:c>
-      <x:c r="D14" s="423" t="str"/>
+      <x:c r="D14" s="423" t="n">
+        <x:v>19</x:v>
+      </x:c>
       <x:c r="E14" s="423" t="n">
         <x:f>COUNTIF('Support - Ledger'!$K$5:$K$304,B14)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F14" s="480" t="str"/>
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="F14" s="480" t="n">
+        <x:v>513.2</x:v>
+      </x:c>
       <x:c r="G14" s="480" t="n">
         <x:f>SUMIF('Support - Ledger'!$K$5:$K$304,B14,'Support - Ledger'!$D$5:$D$304)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H14" s="423" t="str"/>
+        <x:v>513.2</x:v>
+      </x:c>
+      <x:c r="H14" s="423" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
       <x:c r="I14" s="423" t="str">
         <x:f>IF(D14="","Needed",IF(COUNTIFS('Support - Ledger'!$K$5:$K$304,B14,'Support - Ledger'!$M$5:$M$304,"Needs verification")&gt;0,"Needs classification",IF(E14&lt;&gt;D14,"Missing entry",IF(ABS(G14-F14)&gt;0.005,"Total mismatch",IF(H14&lt;&gt;"Yes","Anchor not reached","Verified")))))</x:f>
-        <x:v>Needed</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="J14" s="423" t="str">
-        <x:v>Capture posted activity through the saved anchor</x:v>
+        <x:v>Posted activity reconciled through Sep. 13</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
@@ -4124,23 +4132,29 @@
       <x:c r="C15" s="423" t="str">
         <x:v>Pending ledger rows</x:v>
       </x:c>
-      <x:c r="D15" s="423" t="str"/>
+      <x:c r="D15" s="423" t="n">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="E15" s="423" t="n">
         <x:f>COUNTIF('Support - Ledger'!$K$5:$K$304,B15)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F15" s="480" t="str"/>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F15" s="480" t="n">
+        <x:v>159.54</x:v>
+      </x:c>
       <x:c r="G15" s="480" t="n">
         <x:f>SUMIF('Support - Ledger'!$K$5:$K$304,B15,'Support - Ledger'!$D$5:$D$304)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H15" s="423" t="str"/>
+        <x:v>159.54</x:v>
+      </x:c>
+      <x:c r="H15" s="423" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
       <x:c r="I15" s="423" t="str">
         <x:f>IF(D15="","Needed",IF(COUNTIFS('Support - Ledger'!$K$5:$K$304,B15,'Support - Ledger'!$M$5:$M$304,"Needs verification")&gt;0,"Needs classification",IF(E15&lt;&gt;D15,"Missing entry",IF(ABS(G15-F15)&gt;0.005,"Total mismatch",IF(H15&lt;&gt;"Yes","Anchor not reached","Verified")))))</x:f>
-        <x:v>Needed</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="J15" s="423" t="str">
-        <x:v>Capture all current pending activity</x:v>
+        <x:v>Eight current pending charges reconciled</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
@@ -4175,7 +4189,7 @@
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J16" s="423" t="str">
-        <x:v>Two transactions need category confirmation</x:v>
+        <x:v>All five current rows classified</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
@@ -4245,10 +4259,10 @@
       <x:c r="G19" s="423" t="str"/>
       <x:c r="H19" s="423" t="str"/>
       <x:c r="I19" s="423" t="str">
-        <x:v>Needed</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="J19" s="423" t="str">
-        <x:v>Capture current balance and activity</x:v>
+        <x:v>Current balance $0.00 captured</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="30" customHeight="1">
@@ -4267,10 +4281,10 @@
       <x:c r="G20" s="423" t="str"/>
       <x:c r="H20" s="423" t="str"/>
       <x:c r="I20" s="423" t="str">
-        <x:v>Needed</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="J20" s="423" t="str">
-        <x:v>Capture current balance, activity, and active promo list</x:v>
+        <x:v>All active promo balances captured</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="30" customHeight="1">
@@ -5584,7 +5598,7 @@
     <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="458" t="str">
         <x:f>COUNTIF('1. Start'!E6:E13,"Verified")&amp;" of "&amp;(COUNTA('1. Start'!F6:F14)-COUNTIF('1. Start'!E6:E14,"Not due"))&amp;" source sets verified"</x:f>
-        <x:v>2 of 8 source sets verified</x:v>
+        <x:v>6 of 8 source sets verified</x:v>
       </x:c>
       <x:c r="B6" s="458" t="str">
         <x:v>Sep 1–Sep 7 purchases</x:v>
@@ -5759,7 +5773,7 @@
       </x:c>
       <x:c r="D14" s="468" t="n">
         <x:f>'Support - Promo Detail'!F12</x:f>
-        <x:v>148.616</x:v>
+        <x:v>148.615</x:v>
       </x:c>
       <x:c r="E14" s="460" t="str">
         <x:v>☑ Done</x:v>
@@ -5922,7 +5936,7 @@
       </x:c>
       <x:c r="D21" s="468" t="n">
         <x:f>MAX(0,E23+E25-E24)</x:f>
-        <x:v>48.26999999999998</x:v>
+        <x:v>48.269000000000005</x:v>
       </x:c>
       <x:c r="E21" s="460" t="str">
         <x:v>☐ Pay now</x:v>
@@ -5943,7 +5957,7 @@
       <x:c r="C22" s="458"/>
       <x:c r="D22" s="462" t="n">
         <x:f>SUM(D9:D16,D18:D20)</x:f>
-        <x:v>1275.05</x:v>
+        <x:v>1275.049</x:v>
       </x:c>
       <x:c r="E22" s="423"/>
       <x:c r="F22" s="423"/>
@@ -5958,7 +5972,7 @@
       <x:c r="D23" s="463"/>
       <x:c r="E23" s="469" t="n">
         <x:f>SUM(D9:D16,D18:D20)</x:f>
-        <x:v>1275.05</x:v>
+        <x:v>1275.049</x:v>
       </x:c>
       <x:c r="F23" s="423"/>
       <x:c r="G23" s="423"/>
@@ -5998,7 +6012,7 @@
       <x:c r="D26" s="463"/>
       <x:c r="E26" s="471" t="n">
         <x:f>D21</x:f>
-        <x:v>48.26999999999998</x:v>
+        <x:v>48.269000000000005</x:v>
       </x:c>
       <x:c r="F26" s="423"/>
       <x:c r="G26" s="423"/>
@@ -6072,7 +6086,7 @@
         <x:v>Week beginning (Tuesday)</x:v>
       </x:c>
       <x:c r="B3" s="478" t="n">
-        <x:v>46266</x:v>
+        <x:v>46273</x:v>
       </x:c>
       <x:c r="C3" s="423"/>
       <x:c r="D3" s="423" t="str">
@@ -6080,14 +6094,14 @@
       </x:c>
       <x:c r="E3" s="479" t="n">
         <x:f>B3+6</x:f>
-        <x:v>46272</x:v>
+        <x:v>46279</x:v>
       </x:c>
       <x:c r="F3" s="423" t="str">
         <x:v>Budget status</x:v>
       </x:c>
       <x:c r="G3" s="423" t="str">
         <x:f>IF(COUNTIFS('Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"&lt;&gt;Verified")&gt;0,"Source check needed",IF(F23&lt;0,"Over plan","Within plan"))</x:f>
-        <x:v>Within plan</x:v>
+        <x:v>Over plan</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -6132,7 +6146,7 @@
       </x:c>
       <x:c r="C6" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$F$5:$F$304,A6,'Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$E$5:$E$304,"Posted",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>199.04</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D6" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$F$5:$F$304,A6,'Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$E$5:$E$304,"Pending",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
@@ -6140,15 +6154,15 @@
       </x:c>
       <x:c r="E6" s="480" t="n">
         <x:f>C6+D6</x:f>
-        <x:v>199.04</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F6" s="480" t="n">
         <x:f>IF(B6=0,"",B6-E6)</x:f>
-        <x:v>-119.26307692307692</x:v>
+        <x:v>79.77692307692307</x:v>
       </x:c>
       <x:c r="G6" s="423" t="str">
         <x:f>IF(B6=0,"No target set",IF(E6=0,"No activity",IF(F6&lt;0,"Over plan","On track")))</x:f>
-        <x:v>Over plan</x:v>
+        <x:v>No activity</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="24" customHeight="1">
@@ -6165,19 +6179,19 @@
       </x:c>
       <x:c r="D7" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$F$5:$F$304,A7,'Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$E$5:$E$304,"Pending",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>0</x:v>
+        <x:v>20.91</x:v>
       </x:c>
       <x:c r="E7" s="480" t="n">
         <x:f>C7+D7</x:f>
-        <x:v>0</x:v>
+        <x:v>20.91</x:v>
       </x:c>
       <x:c r="F7" s="480" t="n">
         <x:f>IF(B7=0,"",B7-E7)</x:f>
-        <x:v>25</x:v>
+        <x:v>4.09</x:v>
       </x:c>
       <x:c r="G7" s="423" t="str">
         <x:f>IF(B7=0,"No target set",IF(E7=0,"No activity",IF(F7&lt;0,"Over plan","On track")))</x:f>
-        <x:v>No activity</x:v>
+        <x:v>On track</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="24" customHeight="1">
@@ -6190,19 +6204,19 @@
       </x:c>
       <x:c r="C8" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$F$5:$F$304,A8,'Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$E$5:$E$304,"Posted",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>42.55</x:v>
+        <x:v>39.42</x:v>
       </x:c>
       <x:c r="D8" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$F$5:$F$304,A8,'Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$E$5:$E$304,"Pending",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>0</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E8" s="480" t="n">
         <x:f>C8+D8</x:f>
-        <x:v>42.55</x:v>
+        <x:v>58.42</x:v>
       </x:c>
       <x:c r="F8" s="480" t="n">
         <x:f>IF(B8=0,"",B8-E8)</x:f>
-        <x:v>-12.549999999999997</x:v>
+        <x:v>-28.42</x:v>
       </x:c>
       <x:c r="G8" s="423" t="str">
         <x:f>IF(B8=0,"No target set",IF(E8=0,"No activity",IF(F8&lt;0,"Over plan","On track")))</x:f>
@@ -6219,7 +6233,7 @@
       </x:c>
       <x:c r="C9" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$F$5:$F$304,A9,'Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$E$5:$E$304,"Posted",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>54.56</x:v>
+        <x:v>227.27000000000004</x:v>
       </x:c>
       <x:c r="D9" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$F$5:$F$304,A9,'Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$E$5:$E$304,"Pending",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
@@ -6227,11 +6241,11 @@
       </x:c>
       <x:c r="E9" s="480" t="n">
         <x:f>C9+D9</x:f>
-        <x:v>54.56</x:v>
+        <x:v>227.27000000000004</x:v>
       </x:c>
       <x:c r="F9" s="480" t="n">
         <x:f>IF(B9=0,"",B9-E9)</x:f>
-        <x:v>-4.560000000000002</x:v>
+        <x:v>-177.27000000000004</x:v>
       </x:c>
       <x:c r="G9" s="423" t="str">
         <x:f>IF(B9=0,"No target set",IF(E9=0,"No activity",IF(F9&lt;0,"Over plan","On track")))</x:f>
@@ -6248,23 +6262,23 @@
       </x:c>
       <x:c r="C10" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$F$5:$F$304,A10,'Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$E$5:$E$304,"Posted",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>13.989999999999998</x:v>
+        <x:v>2.82</x:v>
       </x:c>
       <x:c r="D10" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$F$5:$F$304,A10,'Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$E$5:$E$304,"Pending",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>0</x:v>
+        <x:v>2.82</x:v>
       </x:c>
       <x:c r="E10" s="480" t="n">
         <x:f>C10+D10</x:f>
-        <x:v>13.989999999999998</x:v>
+        <x:v>5.64</x:v>
       </x:c>
       <x:c r="F10" s="480" t="n">
         <x:f>IF(B10=0,"",B10-E10)</x:f>
-        <x:v>-3.9899999999999984</x:v>
+        <x:v>4.36</x:v>
       </x:c>
       <x:c r="G10" s="423" t="str">
         <x:f>IF(B10=0,"No target set",IF(E10=0,"No activity",IF(F10&lt;0,"Over plan","On track")))</x:f>
-        <x:v>Over plan</x:v>
+        <x:v>On track</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
@@ -6277,7 +6291,7 @@
       </x:c>
       <x:c r="C11" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$F$5:$F$304,A11,'Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$E$5:$E$304,"Posted",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>-71.46</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D11" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$F$5:$F$304,A11,'Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$E$5:$E$304,"Pending",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
@@ -6285,15 +6299,15 @@
       </x:c>
       <x:c r="E11" s="480" t="n">
         <x:f>C11+D11</x:f>
-        <x:v>-71.46</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F11" s="480" t="n">
         <x:f>IF(B11=0,"",B11-E11)</x:f>
-        <x:v>121.46</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="G11" s="423" t="str">
         <x:f>IF(B11=0,"No target set",IF(E11=0,"No activity",IF(F11&lt;0,"Over plan","On track")))</x:f>
-        <x:v>On track</x:v>
+        <x:v>No activity</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
@@ -6335,19 +6349,19 @@
       </x:c>
       <x:c r="C13" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$F$5:$F$304,A13,'Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$E$5:$E$304,"Posted",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>159.14000000000001</x:v>
+        <x:v>109.84</x:v>
       </x:c>
       <x:c r="D13" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$F$5:$F$304,A13,'Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$E$5:$E$304,"Pending",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>0</x:v>
+        <x:v>63.79</x:v>
       </x:c>
       <x:c r="E13" s="480" t="n">
         <x:f>C13+D13</x:f>
-        <x:v>159.14000000000001</x:v>
+        <x:v>173.63</x:v>
       </x:c>
       <x:c r="F13" s="480" t="n">
         <x:f>IF(B13=0,"",B13-E13)</x:f>
-        <x:v>-78.37076923076924</x:v>
+        <x:v>-92.86076923076922</x:v>
       </x:c>
       <x:c r="G13" s="423" t="str">
         <x:f>IF(B13=0,"No target set",IF(E13=0,"No activity",IF(F13&lt;0,"Over plan","On track")))</x:f>
@@ -6368,19 +6382,19 @@
       </x:c>
       <x:c r="D14" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$F$5:$F$304,A14,'Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$E$5:$E$304,"Pending",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>0</x:v>
+        <x:v>48.27</x:v>
       </x:c>
       <x:c r="E14" s="480" t="n">
         <x:f>C14+D14</x:f>
-        <x:v>0</x:v>
+        <x:v>48.27</x:v>
       </x:c>
       <x:c r="F14" s="480" t="n">
         <x:f>IF(B14=0,"",B14-E14)</x:f>
-        <x:v>47.48076923076923</x:v>
+        <x:v>-0.7892307692307696</x:v>
       </x:c>
       <x:c r="G14" s="423" t="str">
         <x:f>IF(B14=0,"No target set",IF(E14=0,"No activity",IF(F14&lt;0,"Over plan","On track")))</x:f>
-        <x:v>No activity</x:v>
+        <x:v>Over plan</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
@@ -6451,7 +6465,7 @@
       </x:c>
       <x:c r="C17" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$F$5:$F$304,A17,'Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$E$5:$E$304,"Posted",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>35</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D17" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$F$5:$F$304,A17,'Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$E$5:$E$304,"Pending",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
@@ -6459,15 +6473,15 @@
       </x:c>
       <x:c r="E17" s="480" t="n">
         <x:f>C17+D17</x:f>
-        <x:v>35</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F17" s="480" t="n">
         <x:f>IF(B17=0,"",B17-E17)</x:f>
-        <x:v>-13.307692307692307</x:v>
+        <x:v>21.692307692307693</x:v>
       </x:c>
       <x:c r="G17" s="423" t="str">
         <x:f>IF(B17=0,"No target set",IF(E17=0,"No activity",IF(F17&lt;0,"Over plan","On track")))</x:f>
-        <x:v>Over plan</x:v>
+        <x:v>No activity</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
@@ -6480,7 +6494,7 @@
       </x:c>
       <x:c r="C18" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$F$5:$F$304,A18,'Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$E$5:$E$304,"Posted",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>11.99</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D18" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$F$5:$F$304,A18,'Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$E$5:$E$304,"Pending",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
@@ -6488,15 +6502,15 @@
       </x:c>
       <x:c r="E18" s="480" t="n">
         <x:f>C18+D18</x:f>
-        <x:v>11.99</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F18" s="480" t="n">
         <x:f>IF(B18=0,"",B18-E18)</x:f>
-        <x:v>-0.7330769230769238</x:v>
+        <x:v>11.256923076923076</x:v>
       </x:c>
       <x:c r="G18" s="423" t="str">
         <x:f>IF(B18=0,"No target set",IF(E18=0,"No activity",IF(F18&lt;0,"Over plan","On track")))</x:f>
-        <x:v>Over plan</x:v>
+        <x:v>No activity</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="24" customHeight="1">
@@ -6509,15 +6523,15 @@
       </x:c>
       <x:c r="C19" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$F$5:$F$304,A19,'Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$E$5:$E$304,"Posted",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>3</x:v>
+        <x:v>11.99</x:v>
       </x:c>
       <x:c r="D19" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$F$5:$F$304,A19,'Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$E$5:$E$304,"Pending",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>2.5</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E19" s="480" t="n">
         <x:f>C19+D19</x:f>
-        <x:v>5.5</x:v>
+        <x:v>11.99</x:v>
       </x:c>
       <x:c r="F19" s="480" t="str">
         <x:f>IF(B19=0,"",B19-E19)</x:f>
@@ -6537,7 +6551,7 @@
       </x:c>
       <x:c r="C20" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$F$5:$F$304,A20,'Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$E$5:$E$304,"Posted",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>0.18</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D20" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$F$5:$F$304,A20,'Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$E$5:$E$304,"Pending",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
@@ -6545,7 +6559,7 @@
       </x:c>
       <x:c r="E20" s="480" t="n">
         <x:f>C20+D20</x:f>
-        <x:v>0.18</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F20" s="480" t="str">
         <x:f>IF(B20=0,"",B20-E20)</x:f>
@@ -6602,19 +6616,19 @@
       </x:c>
       <x:c r="C23" s="482" t="n">
         <x:f>SUM(C6:C21)</x:f>
-        <x:v>447.99000000000007</x:v>
+        <x:v>391.34000000000003</x:v>
       </x:c>
       <x:c r="D23" s="482" t="n">
         <x:f>SUM(D6:D21)</x:f>
-        <x:v>2.5</x:v>
+        <x:v>154.79</x:v>
       </x:c>
       <x:c r="E23" s="482" t="n">
         <x:f>SUM(E6:E21)</x:f>
-        <x:v>450.49000000000007</x:v>
+        <x:v>546.13</x:v>
       </x:c>
       <x:c r="F23" s="482" t="n">
         <x:f>B23-E23</x:f>
-        <x:v>26.170769230769224</x:v>
+        <x:v>-69.4692307692307</x:v>
       </x:c>
       <x:c r="G23" s="481"/>
     </x:row>
@@ -6900,7 +6914,7 @@
       </x:c>
       <x:c r="B15" s="480" t="n">
         <x:f>'Support - Promo Detail'!F12</x:f>
-        <x:v>148.616</x:v>
+        <x:v>148.615</x:v>
       </x:c>
       <x:c r="C15" s="423" t="str">
         <x:v>Pay weekly</x:v>
@@ -7036,7 +7050,7 @@
       </x:c>
       <x:c r="B23" s="508" t="n">
         <x:f>SUM(B5:B22)</x:f>
-        <x:v>1531.6146692307693</x:v>
+        <x:v>1531.6136692307691</x:v>
       </x:c>
       <x:c r="C23" s="481"/>
       <x:c r="D23" s="481"/>
@@ -7096,7 +7110,7 @@
       </x:c>
       <x:c r="B28" s="512" t="n">
         <x:f>B27-B23</x:f>
-        <x:v>-188.24466923076943</x:v>
+        <x:v>-188.24366923076923</x:v>
       </x:c>
       <x:c r="C28" s="502"/>
       <x:c r="D28" s="503"/>
@@ -7311,7 +7325,7 @@
       </x:c>
       <x:c r="B5" s="562" t="n">
         <x:f>'Support - Account Snapshots'!F6</x:f>
-        <x:v>11847.64</x:v>
+        <x:v>12026.13</x:v>
       </x:c>
       <x:c r="C5" s="539" t="str">
         <x:v>Next rent due</x:v>
@@ -7347,7 +7361,7 @@
       </x:c>
       <x:c r="B7" s="564" t="n">
         <x:f>SUM(B5:B6)</x:f>
-        <x:v>12067.64</x:v>
+        <x:v>12246.13</x:v>
       </x:c>
       <x:c r="C7" s="541" t="str">
         <x:v>Tagged rent reserve</x:v>
@@ -7365,7 +7379,7 @@
       </x:c>
       <x:c r="B8" s="565" t="n">
         <x:f>SUM('Support - Budget Inputs'!E12:E17,'Support - Budget Inputs'!E20:E23,'Support - Budget Inputs'!E25:E26)*13</x:f>
-        <x:v>11985.970700000002</x:v>
+        <x:v>11985.957700000003</x:v>
       </x:c>
       <x:c r="C8" s="541" t="str">
         <x:v>Emergency draw if no more funding</x:v>
@@ -7383,7 +7397,7 @@
       </x:c>
       <x:c r="B9" s="566" t="n">
         <x:f>B7-B8</x:f>
-        <x:v>81.66929999999775</x:v>
+        <x:v>260.17229999999654</x:v>
       </x:c>
       <x:c r="C9" s="545" t="str">
         <x:v>Confirmed funding vs. monthly plan</x:v>
@@ -7537,7 +7551,7 @@
       </x:c>
       <x:c r="B20" s="538" t="n">
         <x:f>'Support - Promo Detail'!C11</x:f>
-        <x:v>1318.93</x:v>
+        <x:v>1170.31</x:v>
       </x:c>
       <x:c r="C20" s="527" t="str">
         <x:v>The weekly payoff is an expense paid from Wells, not savings. The detailed promo schedule is on Support - Promo Detail.</x:v>
@@ -7552,7 +7566,7 @@
       </x:c>
       <x:c r="B21" s="542" t="n">
         <x:f>'Support - Promo Detail'!F12</x:f>
-        <x:v>148.616</x:v>
+        <x:v>148.615</x:v>
       </x:c>
       <x:c r="C21" s="527"/>
       <x:c r="D21" s="527"/>
@@ -8105,15 +8119,15 @@
       <x:c r="H7" s="547"/>
       <x:c r="I7" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$H$5:$H$304,B7,'Support - Ledger'!$E$5:$E$304,"Posted",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>106.26</x:v>
+        <x:v>414.81</x:v>
       </x:c>
       <x:c r="J7" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$H$5:$H$304,B7,'Support - Ledger'!$E$5:$E$304,"Pending",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>138.28</x:v>
+        <x:v>154.79</x:v>
       </x:c>
       <x:c r="K7" s="480" t="n">
         <x:f>I7+J7</x:f>
-        <x:v>244.54000000000002</x:v>
+        <x:v>569.6</x:v>
       </x:c>
       <x:c r="L7" s="480" t="str">
         <x:f>IF(H7="","",H7-K7)</x:f>
@@ -8143,11 +8157,11 @@
       </x:c>
       <x:c r="J8" s="480" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$H$5:$H$304,B8,'Support - Ledger'!$E$5:$E$304,"Pending",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>0</x:v>
+        <x:v>116.80999999999999</x:v>
       </x:c>
       <x:c r="K8" s="480" t="n">
         <x:f>I8+J8</x:f>
-        <x:v>0</x:v>
+        <x:v>116.80999999999999</x:v>
       </x:c>
       <x:c r="L8" s="480" t="str">
         <x:f>IF(H8="","",H8-K8)</x:f>
@@ -11525,7 +11539,7 @@
         <x:v>471.61</x:v>
       </x:c>
       <x:c r="E64" s="548" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Posted</x:v>
       </x:c>
       <x:c r="F64" s="548" t="str">
         <x:v>Emergency car repair</x:v>
@@ -11541,13 +11555,13 @@
         <x:v>chase-2026-09-08-mcwhorter-47161</x:v>
       </x:c>
       <x:c r="J64" s="548" t="str">
-        <x:v>Emergency expense; tracked separately from core scorecard</x:v>
+        <x:v>Posted Sep. 15; emergency repair excluded from core scorecard</x:v>
       </x:c>
       <x:c r="K64" s="548" t="str">
-        <x:v>Chase pending — Sep 9</x:v>
+        <x:v>Chase activity — Sep 15</x:v>
       </x:c>
       <x:c r="L64" s="548" t="str">
-        <x:v>Pending list</x:v>
+        <x:v>Posted activity</x:v>
       </x:c>
       <x:c r="M64" s="548" t="str">
         <x:v>Verified</x:v>
@@ -11567,7 +11581,7 @@
         <x:v>12.45</x:v>
       </x:c>
       <x:c r="E65" s="548" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Posted</x:v>
       </x:c>
       <x:c r="F65" s="548" t="str">
         <x:v>Starbucks</x:v>
@@ -11583,13 +11597,13 @@
         <x:v>chase-2026-09-08-starbucks-1245</x:v>
       </x:c>
       <x:c r="J65" s="548" t="str">
-        <x:v>Pending in Sep. 9 Chase activity</x:v>
+        <x:v>Posted in Sep. 15 Chase activity</x:v>
       </x:c>
       <x:c r="K65" s="548" t="str">
-        <x:v>Chase pending — Sep 9</x:v>
+        <x:v>Chase activity — Sep 15</x:v>
       </x:c>
       <x:c r="L65" s="548" t="str">
-        <x:v>Pending list</x:v>
+        <x:v>Posted activity</x:v>
       </x:c>
       <x:c r="M65" s="548" t="str">
         <x:v>Verified</x:v>
@@ -11609,7 +11623,7 @@
         <x:v>7.22</x:v>
       </x:c>
       <x:c r="E66" s="548" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Posted</x:v>
       </x:c>
       <x:c r="F66" s="548" t="str">
         <x:v>Starbucks</x:v>
@@ -11625,13 +11639,13 @@
         <x:v>chase-2026-09-09-starbucks-722</x:v>
       </x:c>
       <x:c r="J66" s="548" t="str">
-        <x:v>Pending in Sep. 9 Chase activity</x:v>
+        <x:v>Posted in Sep. 15 Chase activity</x:v>
       </x:c>
       <x:c r="K66" s="548" t="str">
-        <x:v>Chase pending — Sep 9</x:v>
+        <x:v>Chase activity — Sep 15</x:v>
       </x:c>
       <x:c r="L66" s="548" t="str">
-        <x:v>Pending list</x:v>
+        <x:v>Posted activity</x:v>
       </x:c>
       <x:c r="M66" s="548" t="str">
         <x:v>Verified</x:v>
@@ -11651,7 +11665,7 @@
         <x:v>6.55</x:v>
       </x:c>
       <x:c r="E67" s="548" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Posted</x:v>
       </x:c>
       <x:c r="F67" s="548" t="str">
         <x:v>Starbucks</x:v>
@@ -11667,13 +11681,13 @@
         <x:v>chase-2026-09-09-starbucks-655</x:v>
       </x:c>
       <x:c r="J67" s="548" t="str">
-        <x:v>Pending in Sep. 9 Chase activity</x:v>
+        <x:v>Posted in Sep. 15 Chase activity</x:v>
       </x:c>
       <x:c r="K67" s="548" t="str">
-        <x:v>Chase pending — Sep 9</x:v>
+        <x:v>Chase activity — Sep 15</x:v>
       </x:c>
       <x:c r="L67" s="548" t="str">
-        <x:v>Pending list</x:v>
+        <x:v>Posted activity</x:v>
       </x:c>
       <x:c r="M67" s="548" t="str">
         <x:v>Verified</x:v>
@@ -12310,395 +12324,970 @@
       </x:c>
     </x:row>
     <x:row r="83">
-      <x:c r="A83" s="548"/>
-      <x:c r="B83" s="478"/>
-      <x:c r="C83" s="548"/>
-      <x:c r="D83" s="547"/>
-      <x:c r="E83" s="548"/>
-      <x:c r="F83" s="548"/>
-      <x:c r="G83" s="548"/>
-      <x:c r="H83" s="574" t="str">
+      <x:c r="A83" s="548" t="str">
+        <x:v>Chase</x:v>
+      </x:c>
+      <x:c r="B83" s="478" t="n">
+        <x:v>46275</x:v>
+      </x:c>
+      <x:c r="C83" s="548" t="str">
+        <x:v>365 MARKET N 888 432-3299</x:v>
+      </x:c>
+      <x:c r="D83" s="547" t="n">
+        <x:v>2.82</x:v>
+      </x:c>
+      <x:c r="E83" s="548" t="str">
+        <x:v>Posted</x:v>
+      </x:c>
+      <x:c r="F83" s="548" t="str">
+        <x:v>Work snacks</x:v>
+      </x:c>
+      <x:c r="G83" s="548" t="str">
+        <x:v>Include</x:v>
+      </x:c>
+      <x:c r="H83" s="574" t="n">
         <x:f>IF(B83="","",B83-WEEKDAY(B83-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I83" s="548"/>
-      <x:c r="J83" s="548"/>
-      <x:c r="K83" s="548"/>
-      <x:c r="L83" s="548"/>
-      <x:c r="M83" s="548"/>
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="I83" s="548" t="str">
+        <x:v>chase-2026-09-10-365-282</x:v>
+      </x:c>
+      <x:c r="J83" s="548" t="str">
+        <x:v>Posted in Sep. 15 Chase activity</x:v>
+      </x:c>
+      <x:c r="K83" s="548" t="str">
+        <x:v>Chase activity — Sep 15</x:v>
+      </x:c>
+      <x:c r="L83" s="548" t="str">
+        <x:v>Posted activity</x:v>
+      </x:c>
+      <x:c r="M83" s="548" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
     </x:row>
     <x:row r="84">
-      <x:c r="A84" s="548"/>
-      <x:c r="B84" s="478"/>
-      <x:c r="C84" s="548"/>
-      <x:c r="D84" s="547"/>
-      <x:c r="E84" s="548"/>
-      <x:c r="F84" s="548"/>
-      <x:c r="G84" s="548"/>
-      <x:c r="H84" s="574" t="str">
+      <x:c r="A84" s="548" t="str">
+        <x:v>Chase</x:v>
+      </x:c>
+      <x:c r="B84" s="478" t="n">
+        <x:v>46275</x:v>
+      </x:c>
+      <x:c r="C84" s="548" t="str">
+        <x:v>PAYMENT THANK YOU</x:v>
+      </x:c>
+      <x:c r="D84" s="547" t="n">
+        <x:v>-266.96</x:v>
+      </x:c>
+      <x:c r="E84" s="548" t="str">
+        <x:v>Posted</x:v>
+      </x:c>
+      <x:c r="F84" s="548" t="str">
+        <x:v>Credit-card payment</x:v>
+      </x:c>
+      <x:c r="G84" s="548" t="str">
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="H84" s="574" t="n">
         <x:f>IF(B84="","",B84-WEEKDAY(B84-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I84" s="548"/>
-      <x:c r="J84" s="548"/>
-      <x:c r="K84" s="548"/>
-      <x:c r="L84" s="548"/>
-      <x:c r="M84" s="548"/>
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="I84" s="548" t="str">
+        <x:v>chase-2026-09-10-payment-26696</x:v>
+      </x:c>
+      <x:c r="J84" s="548" t="str">
+        <x:v>Payment also confirmed by Wells; excluded from spending</x:v>
+      </x:c>
+      <x:c r="K84" s="548" t="str">
+        <x:v>Chase activity — Sep 15</x:v>
+      </x:c>
+      <x:c r="L84" s="548" t="str">
+        <x:v>Posted activity</x:v>
+      </x:c>
+      <x:c r="M84" s="548" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
     </x:row>
     <x:row r="85">
-      <x:c r="A85" s="548"/>
-      <x:c r="B85" s="478"/>
-      <x:c r="C85" s="548"/>
-      <x:c r="D85" s="547"/>
-      <x:c r="E85" s="548"/>
-      <x:c r="F85" s="548"/>
-      <x:c r="G85" s="548"/>
-      <x:c r="H85" s="574" t="str">
+      <x:c r="A85" s="548" t="str">
+        <x:v>Chase</x:v>
+      </x:c>
+      <x:c r="B85" s="478" t="n">
+        <x:v>46275</x:v>
+      </x:c>
+      <x:c r="C85" s="548" t="str">
+        <x:v>INVINCIBLE APPCHARGE</x:v>
+      </x:c>
+      <x:c r="D85" s="547" t="n">
+        <x:v>27.53</x:v>
+      </x:c>
+      <x:c r="E85" s="548" t="str">
+        <x:v>Posted</x:v>
+      </x:c>
+      <x:c r="F85" s="548" t="str">
+        <x:v>Invincibles + other Apple</x:v>
+      </x:c>
+      <x:c r="G85" s="548" t="str">
+        <x:v>Include</x:v>
+      </x:c>
+      <x:c r="H85" s="574" t="n">
         <x:f>IF(B85="","",B85-WEEKDAY(B85-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I85" s="548"/>
-      <x:c r="J85" s="548"/>
-      <x:c r="K85" s="548"/>
-      <x:c r="L85" s="548"/>
-      <x:c r="M85" s="548"/>
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="I85" s="548" t="str">
+        <x:v>chase-2026-09-10-invincible-2753</x:v>
+      </x:c>
+      <x:c r="J85" s="548" t="str">
+        <x:v>Posted in Sep. 15 Chase activity</x:v>
+      </x:c>
+      <x:c r="K85" s="548" t="str">
+        <x:v>Chase activity — Sep 15</x:v>
+      </x:c>
+      <x:c r="L85" s="548" t="str">
+        <x:v>Posted activity</x:v>
+      </x:c>
+      <x:c r="M85" s="548" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
     </x:row>
     <x:row r="86">
-      <x:c r="A86" s="548"/>
-      <x:c r="B86" s="478"/>
-      <x:c r="C86" s="548"/>
-      <x:c r="D86" s="547"/>
-      <x:c r="E86" s="548"/>
-      <x:c r="F86" s="548"/>
-      <x:c r="G86" s="548"/>
-      <x:c r="H86" s="574" t="str">
+      <x:c r="A86" s="548" t="str">
+        <x:v>Chase</x:v>
+      </x:c>
+      <x:c r="B86" s="478" t="n">
+        <x:v>46275</x:v>
+      </x:c>
+      <x:c r="C86" s="548" t="str">
+        <x:v>APPLE DIGITAL SERVICES</x:v>
+      </x:c>
+      <x:c r="D86" s="547" t="n">
+        <x:v>16.21</x:v>
+      </x:c>
+      <x:c r="E86" s="548" t="str">
+        <x:v>Posted</x:v>
+      </x:c>
+      <x:c r="F86" s="548" t="str">
+        <x:v>Invincibles + other Apple</x:v>
+      </x:c>
+      <x:c r="G86" s="548" t="str">
+        <x:v>Include</x:v>
+      </x:c>
+      <x:c r="H86" s="574" t="n">
         <x:f>IF(B86="","",B86-WEEKDAY(B86-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I86" s="548"/>
-      <x:c r="J86" s="548"/>
-      <x:c r="K86" s="548"/>
-      <x:c r="L86" s="548"/>
-      <x:c r="M86" s="548"/>
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="I86" s="548" t="str">
+        <x:v>chase-2026-09-10-apple-1621</x:v>
+      </x:c>
+      <x:c r="J86" s="548" t="str">
+        <x:v>Posted in Sep. 15 Chase activity</x:v>
+      </x:c>
+      <x:c r="K86" s="548" t="str">
+        <x:v>Chase activity — Sep 15</x:v>
+      </x:c>
+      <x:c r="L86" s="548" t="str">
+        <x:v>Posted activity</x:v>
+      </x:c>
+      <x:c r="M86" s="548" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
     </x:row>
     <x:row r="87">
-      <x:c r="A87" s="548"/>
-      <x:c r="B87" s="478"/>
-      <x:c r="C87" s="548"/>
-      <x:c r="D87" s="547"/>
-      <x:c r="E87" s="548"/>
-      <x:c r="F87" s="548"/>
-      <x:c r="G87" s="548"/>
-      <x:c r="H87" s="574" t="str">
+      <x:c r="A87" s="548" t="str">
+        <x:v>Chase</x:v>
+      </x:c>
+      <x:c r="B87" s="478" t="n">
+        <x:v>46275</x:v>
+      </x:c>
+      <x:c r="C87" s="548" t="str">
+        <x:v>INVINCIBLE APPCHARGE</x:v>
+      </x:c>
+      <x:c r="D87" s="547" t="n">
+        <x:v>13.76</x:v>
+      </x:c>
+      <x:c r="E87" s="548" t="str">
+        <x:v>Posted</x:v>
+      </x:c>
+      <x:c r="F87" s="548" t="str">
+        <x:v>Invincibles + other Apple</x:v>
+      </x:c>
+      <x:c r="G87" s="548" t="str">
+        <x:v>Include</x:v>
+      </x:c>
+      <x:c r="H87" s="574" t="n">
         <x:f>IF(B87="","",B87-WEEKDAY(B87-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I87" s="548"/>
-      <x:c r="J87" s="548"/>
-      <x:c r="K87" s="548"/>
-      <x:c r="L87" s="548"/>
-      <x:c r="M87" s="548"/>
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="I87" s="548" t="str">
+        <x:v>chase-2026-09-10-invincible-1376</x:v>
+      </x:c>
+      <x:c r="J87" s="548" t="str">
+        <x:v>Posted in Sep. 15 Chase activity</x:v>
+      </x:c>
+      <x:c r="K87" s="548" t="str">
+        <x:v>Chase activity — Sep 15</x:v>
+      </x:c>
+      <x:c r="L87" s="548" t="str">
+        <x:v>Posted activity</x:v>
+      </x:c>
+      <x:c r="M87" s="548" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
     </x:row>
     <x:row r="88">
-      <x:c r="A88" s="548"/>
-      <x:c r="B88" s="478"/>
-      <x:c r="C88" s="548"/>
-      <x:c r="D88" s="547"/>
-      <x:c r="E88" s="548"/>
-      <x:c r="F88" s="548"/>
-      <x:c r="G88" s="548"/>
-      <x:c r="H88" s="574" t="str">
+      <x:c r="A88" s="548" t="str">
+        <x:v>Chase</x:v>
+      </x:c>
+      <x:c r="B88" s="478" t="n">
+        <x:v>46275</x:v>
+      </x:c>
+      <x:c r="C88" s="548" t="str">
+        <x:v>INVINCIBLE APPCHARGE</x:v>
+      </x:c>
+      <x:c r="D88" s="547" t="n">
+        <x:v>4.58</x:v>
+      </x:c>
+      <x:c r="E88" s="548" t="str">
+        <x:v>Posted</x:v>
+      </x:c>
+      <x:c r="F88" s="548" t="str">
+        <x:v>Invincibles + other Apple</x:v>
+      </x:c>
+      <x:c r="G88" s="548" t="str">
+        <x:v>Include</x:v>
+      </x:c>
+      <x:c r="H88" s="574" t="n">
         <x:f>IF(B88="","",B88-WEEKDAY(B88-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I88" s="548"/>
-      <x:c r="J88" s="548"/>
-      <x:c r="K88" s="548"/>
-      <x:c r="L88" s="548"/>
-      <x:c r="M88" s="548"/>
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="I88" s="548" t="str">
+        <x:v>chase-2026-09-10-invincible-458</x:v>
+      </x:c>
+      <x:c r="J88" s="548" t="str">
+        <x:v>Posted in Sep. 15 Chase activity</x:v>
+      </x:c>
+      <x:c r="K88" s="548" t="str">
+        <x:v>Chase activity — Sep 15</x:v>
+      </x:c>
+      <x:c r="L88" s="548" t="str">
+        <x:v>Posted activity</x:v>
+      </x:c>
+      <x:c r="M88" s="548" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
     </x:row>
     <x:row r="89">
-      <x:c r="A89" s="548"/>
-      <x:c r="B89" s="478"/>
-      <x:c r="C89" s="548"/>
-      <x:c r="D89" s="547"/>
-      <x:c r="E89" s="548"/>
-      <x:c r="F89" s="548"/>
-      <x:c r="G89" s="548"/>
-      <x:c r="H89" s="574" t="str">
+      <x:c r="A89" s="548" t="str">
+        <x:v>Chase</x:v>
+      </x:c>
+      <x:c r="B89" s="478" t="n">
+        <x:v>46276</x:v>
+      </x:c>
+      <x:c r="C89" s="548" t="str">
+        <x:v>EXXON</x:v>
+      </x:c>
+      <x:c r="D89" s="547" t="n">
+        <x:v>27.05</x:v>
+      </x:c>
+      <x:c r="E89" s="548" t="str">
+        <x:v>Posted</x:v>
+      </x:c>
+      <x:c r="F89" s="548" t="str">
+        <x:v>Fuel</x:v>
+      </x:c>
+      <x:c r="G89" s="548" t="str">
+        <x:v>Include</x:v>
+      </x:c>
+      <x:c r="H89" s="574" t="n">
         <x:f>IF(B89="","",B89-WEEKDAY(B89-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I89" s="548"/>
-      <x:c r="J89" s="548"/>
-      <x:c r="K89" s="548"/>
-      <x:c r="L89" s="548"/>
-      <x:c r="M89" s="548"/>
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="I89" s="548" t="str">
+        <x:v>chase-2026-09-11-exxon-2705</x:v>
+      </x:c>
+      <x:c r="J89" s="548" t="str">
+        <x:v>Posted in Sep. 15 Chase activity</x:v>
+      </x:c>
+      <x:c r="K89" s="548" t="str">
+        <x:v>Chase activity — Sep 15</x:v>
+      </x:c>
+      <x:c r="L89" s="548" t="str">
+        <x:v>Posted activity</x:v>
+      </x:c>
+      <x:c r="M89" s="548" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
     </x:row>
     <x:row r="90">
-      <x:c r="A90" s="548"/>
-      <x:c r="B90" s="478"/>
-      <x:c r="C90" s="548"/>
-      <x:c r="D90" s="547"/>
-      <x:c r="E90" s="548"/>
-      <x:c r="F90" s="548"/>
-      <x:c r="G90" s="548"/>
-      <x:c r="H90" s="574" t="str">
+      <x:c r="A90" s="548" t="str">
+        <x:v>Chase</x:v>
+      </x:c>
+      <x:c r="B90" s="478" t="n">
+        <x:v>46276</x:v>
+      </x:c>
+      <x:c r="C90" s="548" t="str">
+        <x:v>INVINCIBLE APPCHARGE</x:v>
+      </x:c>
+      <x:c r="D90" s="547" t="n">
+        <x:v>18.35</x:v>
+      </x:c>
+      <x:c r="E90" s="548" t="str">
+        <x:v>Posted</x:v>
+      </x:c>
+      <x:c r="F90" s="548" t="str">
+        <x:v>Invincibles + other Apple</x:v>
+      </x:c>
+      <x:c r="G90" s="548" t="str">
+        <x:v>Include</x:v>
+      </x:c>
+      <x:c r="H90" s="574" t="n">
         <x:f>IF(B90="","",B90-WEEKDAY(B90-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I90" s="548"/>
-      <x:c r="J90" s="548"/>
-      <x:c r="K90" s="548"/>
-      <x:c r="L90" s="548"/>
-      <x:c r="M90" s="548"/>
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="I90" s="548" t="str">
+        <x:v>chase-2026-09-11-invincible-1835</x:v>
+      </x:c>
+      <x:c r="J90" s="548" t="str">
+        <x:v>Posted in Sep. 15 Chase activity</x:v>
+      </x:c>
+      <x:c r="K90" s="548" t="str">
+        <x:v>Chase activity — Sep 15</x:v>
+      </x:c>
+      <x:c r="L90" s="548" t="str">
+        <x:v>Posted activity</x:v>
+      </x:c>
+      <x:c r="M90" s="548" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
     </x:row>
     <x:row r="91">
-      <x:c r="A91" s="548"/>
-      <x:c r="B91" s="478"/>
-      <x:c r="C91" s="548"/>
-      <x:c r="D91" s="547"/>
-      <x:c r="E91" s="548"/>
-      <x:c r="F91" s="548"/>
-      <x:c r="G91" s="548"/>
-      <x:c r="H91" s="574" t="str">
+      <x:c r="A91" s="548" t="str">
+        <x:v>Chase</x:v>
+      </x:c>
+      <x:c r="B91" s="478" t="n">
+        <x:v>46276</x:v>
+      </x:c>
+      <x:c r="C91" s="548" t="str">
+        <x:v>Starbucks</x:v>
+      </x:c>
+      <x:c r="D91" s="547" t="n">
+        <x:v>6.22</x:v>
+      </x:c>
+      <x:c r="E91" s="548" t="str">
+        <x:v>Posted</x:v>
+      </x:c>
+      <x:c r="F91" s="548" t="str">
+        <x:v>Starbucks</x:v>
+      </x:c>
+      <x:c r="G91" s="548" t="str">
+        <x:v>Include</x:v>
+      </x:c>
+      <x:c r="H91" s="574" t="n">
         <x:f>IF(B91="","",B91-WEEKDAY(B91-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I91" s="548"/>
-      <x:c r="J91" s="548"/>
-      <x:c r="K91" s="548"/>
-      <x:c r="L91" s="548"/>
-      <x:c r="M91" s="548"/>
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="I91" s="548" t="str">
+        <x:v>chase-2026-09-11-starbucks-622</x:v>
+      </x:c>
+      <x:c r="J91" s="548" t="str">
+        <x:v>Posted in Sep. 15 Chase activity</x:v>
+      </x:c>
+      <x:c r="K91" s="548" t="str">
+        <x:v>Chase activity — Sep 15</x:v>
+      </x:c>
+      <x:c r="L91" s="548" t="str">
+        <x:v>Posted activity</x:v>
+      </x:c>
+      <x:c r="M91" s="548" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
     </x:row>
     <x:row r="92">
-      <x:c r="A92" s="548"/>
-      <x:c r="B92" s="478"/>
-      <x:c r="C92" s="548"/>
-      <x:c r="D92" s="547"/>
-      <x:c r="E92" s="548"/>
-      <x:c r="F92" s="548"/>
-      <x:c r="G92" s="548"/>
-      <x:c r="H92" s="574" t="str">
+      <x:c r="A92" s="548" t="str">
+        <x:v>Chase</x:v>
+      </x:c>
+      <x:c r="B92" s="478" t="n">
+        <x:v>46277</x:v>
+      </x:c>
+      <x:c r="C92" s="548" t="str">
+        <x:v>Starbucks</x:v>
+      </x:c>
+      <x:c r="D92" s="547" t="n">
+        <x:v>6.98</x:v>
+      </x:c>
+      <x:c r="E92" s="548" t="str">
+        <x:v>Posted</x:v>
+      </x:c>
+      <x:c r="F92" s="548" t="str">
+        <x:v>Starbucks</x:v>
+      </x:c>
+      <x:c r="G92" s="548" t="str">
+        <x:v>Include</x:v>
+      </x:c>
+      <x:c r="H92" s="574" t="n">
         <x:f>IF(B92="","",B92-WEEKDAY(B92-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I92" s="548"/>
-      <x:c r="J92" s="548"/>
-      <x:c r="K92" s="548"/>
-      <x:c r="L92" s="548"/>
-      <x:c r="M92" s="548"/>
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="I92" s="548" t="str">
+        <x:v>chase-2026-09-12-starbucks-698</x:v>
+      </x:c>
+      <x:c r="J92" s="548" t="str">
+        <x:v>Posted in Sep. 15 Chase activity</x:v>
+      </x:c>
+      <x:c r="K92" s="548" t="str">
+        <x:v>Chase activity — Sep 15</x:v>
+      </x:c>
+      <x:c r="L92" s="548" t="str">
+        <x:v>Posted activity</x:v>
+      </x:c>
+      <x:c r="M92" s="548" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
     </x:row>
     <x:row r="93">
-      <x:c r="A93" s="548"/>
-      <x:c r="B93" s="478"/>
-      <x:c r="C93" s="548"/>
-      <x:c r="D93" s="547"/>
-      <x:c r="E93" s="548"/>
-      <x:c r="F93" s="548"/>
-      <x:c r="G93" s="548"/>
-      <x:c r="H93" s="574" t="str">
+      <x:c r="A93" s="548" t="str">
+        <x:v>Chase</x:v>
+      </x:c>
+      <x:c r="B93" s="478" t="n">
+        <x:v>46277</x:v>
+      </x:c>
+      <x:c r="C93" s="548" t="str">
+        <x:v>INVINCIBLE APPCHARGE</x:v>
+      </x:c>
+      <x:c r="D93" s="547" t="n">
+        <x:v>13.76</x:v>
+      </x:c>
+      <x:c r="E93" s="548" t="str">
+        <x:v>Posted</x:v>
+      </x:c>
+      <x:c r="F93" s="548" t="str">
+        <x:v>Invincibles + other Apple</x:v>
+      </x:c>
+      <x:c r="G93" s="548" t="str">
+        <x:v>Include</x:v>
+      </x:c>
+      <x:c r="H93" s="574" t="n">
         <x:f>IF(B93="","",B93-WEEKDAY(B93-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I93" s="548"/>
-      <x:c r="J93" s="548"/>
-      <x:c r="K93" s="548"/>
-      <x:c r="L93" s="548"/>
-      <x:c r="M93" s="548"/>
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="I93" s="548" t="str">
+        <x:v>chase-2026-09-12-invincible-1376</x:v>
+      </x:c>
+      <x:c r="J93" s="548" t="str">
+        <x:v>Posted in Sep. 15 Chase activity</x:v>
+      </x:c>
+      <x:c r="K93" s="548" t="str">
+        <x:v>Chase activity — Sep 15</x:v>
+      </x:c>
+      <x:c r="L93" s="548" t="str">
+        <x:v>Posted activity</x:v>
+      </x:c>
+      <x:c r="M93" s="548" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
     </x:row>
     <x:row r="94">
-      <x:c r="A94" s="548"/>
-      <x:c r="B94" s="478"/>
-      <x:c r="C94" s="548"/>
-      <x:c r="D94" s="547"/>
-      <x:c r="E94" s="548"/>
-      <x:c r="F94" s="548"/>
-      <x:c r="G94" s="548"/>
-      <x:c r="H94" s="574" t="str">
+      <x:c r="A94" s="548" t="str">
+        <x:v>Chase</x:v>
+      </x:c>
+      <x:c r="B94" s="478" t="n">
+        <x:v>46278</x:v>
+      </x:c>
+      <x:c r="C94" s="548" t="str">
+        <x:v>INVINCIBLE APPCHARGE</x:v>
+      </x:c>
+      <x:c r="D94" s="547" t="n">
+        <x:v>13.76</x:v>
+      </x:c>
+      <x:c r="E94" s="548" t="str">
+        <x:v>Posted</x:v>
+      </x:c>
+      <x:c r="F94" s="548" t="str">
+        <x:v>Invincibles + other Apple</x:v>
+      </x:c>
+      <x:c r="G94" s="548" t="str">
+        <x:v>Include</x:v>
+      </x:c>
+      <x:c r="H94" s="574" t="n">
         <x:f>IF(B94="","",B94-WEEKDAY(B94-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I94" s="548"/>
-      <x:c r="J94" s="548"/>
-      <x:c r="K94" s="548"/>
-      <x:c r="L94" s="548"/>
-      <x:c r="M94" s="548"/>
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="I94" s="548" t="str">
+        <x:v>chase-2026-09-13-invincible-1376</x:v>
+      </x:c>
+      <x:c r="J94" s="548" t="str">
+        <x:v>Posted in Sep. 15 Chase activity</x:v>
+      </x:c>
+      <x:c r="K94" s="548" t="str">
+        <x:v>Chase activity — Sep 15</x:v>
+      </x:c>
+      <x:c r="L94" s="548" t="str">
+        <x:v>Posted activity</x:v>
+      </x:c>
+      <x:c r="M94" s="548" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
     </x:row>
     <x:row r="95">
-      <x:c r="A95" s="548"/>
-      <x:c r="B95" s="478"/>
-      <x:c r="C95" s="548"/>
-      <x:c r="D95" s="547"/>
-      <x:c r="E95" s="548"/>
-      <x:c r="F95" s="548"/>
-      <x:c r="G95" s="548"/>
-      <x:c r="H95" s="574" t="str">
+      <x:c r="A95" s="548" t="str">
+        <x:v>Chase</x:v>
+      </x:c>
+      <x:c r="B95" s="478" t="n">
+        <x:v>46278</x:v>
+      </x:c>
+      <x:c r="C95" s="548" t="str">
+        <x:v>INVINCIBLE APPCHARGE</x:v>
+      </x:c>
+      <x:c r="D95" s="547" t="n">
+        <x:v>27.53</x:v>
+      </x:c>
+      <x:c r="E95" s="548" t="str">
+        <x:v>Posted</x:v>
+      </x:c>
+      <x:c r="F95" s="548" t="str">
+        <x:v>Invincibles + other Apple</x:v>
+      </x:c>
+      <x:c r="G95" s="548" t="str">
+        <x:v>Include</x:v>
+      </x:c>
+      <x:c r="H95" s="574" t="n">
         <x:f>IF(B95="","",B95-WEEKDAY(B95-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I95" s="548"/>
-      <x:c r="J95" s="548"/>
-      <x:c r="K95" s="548"/>
-      <x:c r="L95" s="548"/>
-      <x:c r="M95" s="548"/>
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="I95" s="548" t="str">
+        <x:v>chase-2026-09-13-invincible-2753</x:v>
+      </x:c>
+      <x:c r="J95" s="548" t="str">
+        <x:v>Posted in Sep. 15 Chase activity</x:v>
+      </x:c>
+      <x:c r="K95" s="548" t="str">
+        <x:v>Chase activity — Sep 15</x:v>
+      </x:c>
+      <x:c r="L95" s="548" t="str">
+        <x:v>Posted activity</x:v>
+      </x:c>
+      <x:c r="M95" s="548" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
     </x:row>
     <x:row r="96">
-      <x:c r="A96" s="548"/>
-      <x:c r="B96" s="478"/>
-      <x:c r="C96" s="548"/>
-      <x:c r="D96" s="547"/>
-      <x:c r="E96" s="548"/>
-      <x:c r="F96" s="548"/>
-      <x:c r="G96" s="548"/>
-      <x:c r="H96" s="574" t="str">
+      <x:c r="A96" s="548" t="str">
+        <x:v>Chase</x:v>
+      </x:c>
+      <x:c r="B96" s="478" t="n">
+        <x:v>46278</x:v>
+      </x:c>
+      <x:c r="C96" s="548" t="str">
+        <x:v>ARKPERFORMA</x:v>
+      </x:c>
+      <x:c r="D96" s="547" t="n">
+        <x:v>11.99</x:v>
+      </x:c>
+      <x:c r="E96" s="548" t="str">
+        <x:v>Posted</x:v>
+      </x:c>
+      <x:c r="F96" s="548" t="str">
+        <x:v>Automotive</x:v>
+      </x:c>
+      <x:c r="G96" s="548" t="str">
+        <x:v>Include</x:v>
+      </x:c>
+      <x:c r="H96" s="574" t="n">
         <x:f>IF(B96="","",B96-WEEKDAY(B96-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I96" s="548"/>
-      <x:c r="J96" s="548"/>
-      <x:c r="K96" s="548"/>
-      <x:c r="L96" s="548"/>
-      <x:c r="M96" s="548"/>
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="I96" s="548" t="str">
+        <x:v>chase-2026-09-13-arkperforma-1199</x:v>
+      </x:c>
+      <x:c r="J96" s="548" t="str">
+        <x:v>Same merchant previously classified as automotive</x:v>
+      </x:c>
+      <x:c r="K96" s="548" t="str">
+        <x:v>Chase activity — Sep 15</x:v>
+      </x:c>
+      <x:c r="L96" s="548" t="str">
+        <x:v>Posted activity</x:v>
+      </x:c>
+      <x:c r="M96" s="548" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
     </x:row>
     <x:row r="97">
-      <x:c r="A97" s="548"/>
-      <x:c r="B97" s="478"/>
-      <x:c r="C97" s="548"/>
-      <x:c r="D97" s="547"/>
-      <x:c r="E97" s="548"/>
-      <x:c r="F97" s="548"/>
-      <x:c r="G97" s="548"/>
-      <x:c r="H97" s="574" t="str">
+      <x:c r="A97" s="548" t="str">
+        <x:v>Chase</x:v>
+      </x:c>
+      <x:c r="B97" s="478" t="n">
+        <x:v>46278</x:v>
+      </x:c>
+      <x:c r="C97" s="548" t="str">
+        <x:v>INVINCIBLE APPCHARGE</x:v>
+      </x:c>
+      <x:c r="D97" s="547" t="n">
+        <x:v>91.79</x:v>
+      </x:c>
+      <x:c r="E97" s="548" t="str">
+        <x:v>Posted</x:v>
+      </x:c>
+      <x:c r="F97" s="548" t="str">
+        <x:v>Invincibles + other Apple</x:v>
+      </x:c>
+      <x:c r="G97" s="548" t="str">
+        <x:v>Include</x:v>
+      </x:c>
+      <x:c r="H97" s="574" t="n">
         <x:f>IF(B97="","",B97-WEEKDAY(B97-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I97" s="548"/>
-      <x:c r="J97" s="548"/>
-      <x:c r="K97" s="548"/>
-      <x:c r="L97" s="548"/>
-      <x:c r="M97" s="548"/>
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="I97" s="548" t="str">
+        <x:v>chase-2026-09-13-invincible-9179</x:v>
+      </x:c>
+      <x:c r="J97" s="548" t="str">
+        <x:v>Posted in Sep. 15 Chase activity</x:v>
+      </x:c>
+      <x:c r="K97" s="548" t="str">
+        <x:v>Chase activity — Sep 15</x:v>
+      </x:c>
+      <x:c r="L97" s="548" t="str">
+        <x:v>Posted activity</x:v>
+      </x:c>
+      <x:c r="M97" s="548" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
     </x:row>
     <x:row r="98">
-      <x:c r="A98" s="548"/>
-      <x:c r="B98" s="478"/>
-      <x:c r="C98" s="548"/>
-      <x:c r="D98" s="547"/>
-      <x:c r="E98" s="548"/>
-      <x:c r="F98" s="548"/>
-      <x:c r="G98" s="548"/>
-      <x:c r="H98" s="574" t="str">
+      <x:c r="A98" s="548" t="str">
+        <x:v>Chase</x:v>
+      </x:c>
+      <x:c r="B98" s="478" t="n">
+        <x:v>46278</x:v>
+      </x:c>
+      <x:c r="C98" s="548" t="str">
+        <x:v>DOORDASH MCCONALD'S</x:v>
+      </x:c>
+      <x:c r="D98" s="547" t="n">
+        <x:v>20.91</x:v>
+      </x:c>
+      <x:c r="E98" s="548" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="F98" s="548" t="str">
+        <x:v>DoorDash</x:v>
+      </x:c>
+      <x:c r="G98" s="548" t="str">
+        <x:v>Include</x:v>
+      </x:c>
+      <x:c r="H98" s="574" t="n">
         <x:f>IF(B98="","",B98-WEEKDAY(B98-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I98" s="548"/>
-      <x:c r="J98" s="548"/>
-      <x:c r="K98" s="548"/>
-      <x:c r="L98" s="548"/>
-      <x:c r="M98" s="548"/>
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="I98" s="548" t="str">
+        <x:v>chase-2026-09-13-doordash-2091</x:v>
+      </x:c>
+      <x:c r="J98" s="548" t="str">
+        <x:v>Pending in Sep. 15 Chase activity</x:v>
+      </x:c>
+      <x:c r="K98" s="548" t="str">
+        <x:v>Chase pending — Sep 15</x:v>
+      </x:c>
+      <x:c r="L98" s="548" t="str">
+        <x:v>Pending list</x:v>
+      </x:c>
+      <x:c r="M98" s="548" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
     </x:row>
     <x:row r="99">
-      <x:c r="A99" s="548"/>
-      <x:c r="B99" s="478"/>
-      <x:c r="C99" s="548"/>
-      <x:c r="D99" s="547"/>
-      <x:c r="E99" s="548"/>
-      <x:c r="F99" s="548"/>
-      <x:c r="G99" s="548"/>
-      <x:c r="H99" s="574" t="str">
+      <x:c r="A99" s="548" t="str">
+        <x:v>Chase</x:v>
+      </x:c>
+      <x:c r="B99" s="478" t="n">
+        <x:v>46278</x:v>
+      </x:c>
+      <x:c r="C99" s="548" t="str">
+        <x:v>Starbucks</x:v>
+      </x:c>
+      <x:c r="D99" s="547" t="n">
+        <x:v>6.55</x:v>
+      </x:c>
+      <x:c r="E99" s="548" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="F99" s="548" t="str">
+        <x:v>Starbucks</x:v>
+      </x:c>
+      <x:c r="G99" s="548" t="str">
+        <x:v>Include</x:v>
+      </x:c>
+      <x:c r="H99" s="574" t="n">
         <x:f>IF(B99="","",B99-WEEKDAY(B99-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I99" s="548"/>
-      <x:c r="J99" s="548"/>
-      <x:c r="K99" s="548"/>
-      <x:c r="L99" s="548"/>
-      <x:c r="M99" s="548"/>
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="I99" s="548" t="str">
+        <x:v>chase-2026-09-13-starbucks-655</x:v>
+      </x:c>
+      <x:c r="J99" s="548" t="str">
+        <x:v>Pending in Sep. 15 Chase activity</x:v>
+      </x:c>
+      <x:c r="K99" s="548" t="str">
+        <x:v>Chase pending — Sep 15</x:v>
+      </x:c>
+      <x:c r="L99" s="548" t="str">
+        <x:v>Pending list</x:v>
+      </x:c>
+      <x:c r="M99" s="548" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
     </x:row>
     <x:row r="100">
-      <x:c r="A100" s="548"/>
-      <x:c r="B100" s="478"/>
-      <x:c r="C100" s="548"/>
-      <x:c r="D100" s="547"/>
-      <x:c r="E100" s="548"/>
-      <x:c r="F100" s="548"/>
-      <x:c r="G100" s="548"/>
-      <x:c r="H100" s="574" t="str">
+      <x:c r="A100" s="548" t="str">
+        <x:v>Chase</x:v>
+      </x:c>
+      <x:c r="B100" s="478" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="C100" s="548" t="str">
+        <x:v>365 MARKET N 888 432-3299</x:v>
+      </x:c>
+      <x:c r="D100" s="547" t="n">
+        <x:v>2.82</x:v>
+      </x:c>
+      <x:c r="E100" s="548" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="F100" s="548" t="str">
+        <x:v>Work snacks</x:v>
+      </x:c>
+      <x:c r="G100" s="548" t="str">
+        <x:v>Include</x:v>
+      </x:c>
+      <x:c r="H100" s="574" t="n">
         <x:f>IF(B100="","",B100-WEEKDAY(B100-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I100" s="548"/>
-      <x:c r="J100" s="548"/>
-      <x:c r="K100" s="548"/>
-      <x:c r="L100" s="548"/>
-      <x:c r="M100" s="548"/>
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="I100" s="548" t="str">
+        <x:v>chase-2026-09-14-365-282</x:v>
+      </x:c>
+      <x:c r="J100" s="548" t="str">
+        <x:v>Pending in Sep. 15 Chase activity</x:v>
+      </x:c>
+      <x:c r="K100" s="548" t="str">
+        <x:v>Chase pending — Sep 15</x:v>
+      </x:c>
+      <x:c r="L100" s="548" t="str">
+        <x:v>Pending list</x:v>
+      </x:c>
+      <x:c r="M100" s="548" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
     </x:row>
     <x:row r="101">
-      <x:c r="A101" s="548"/>
-      <x:c r="B101" s="478"/>
-      <x:c r="C101" s="548"/>
-      <x:c r="D101" s="547"/>
-      <x:c r="E101" s="548"/>
-      <x:c r="F101" s="548"/>
-      <x:c r="G101" s="548"/>
-      <x:c r="H101" s="574" t="str">
+      <x:c r="A101" s="548" t="str">
+        <x:v>Chase</x:v>
+      </x:c>
+      <x:c r="B101" s="478" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="C101" s="548" t="str">
+        <x:v>Starbucks</x:v>
+      </x:c>
+      <x:c r="D101" s="547" t="n">
+        <x:v>12.45</x:v>
+      </x:c>
+      <x:c r="E101" s="548" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="F101" s="548" t="str">
+        <x:v>Starbucks</x:v>
+      </x:c>
+      <x:c r="G101" s="548" t="str">
+        <x:v>Include</x:v>
+      </x:c>
+      <x:c r="H101" s="574" t="n">
         <x:f>IF(B101="","",B101-WEEKDAY(B101-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I101" s="548"/>
-      <x:c r="J101" s="548"/>
-      <x:c r="K101" s="548"/>
-      <x:c r="L101" s="548"/>
-      <x:c r="M101" s="548"/>
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="I101" s="548" t="str">
+        <x:v>chase-2026-09-14-starbucks-1245</x:v>
+      </x:c>
+      <x:c r="J101" s="548" t="str">
+        <x:v>Pending in Sep. 15 Chase activity</x:v>
+      </x:c>
+      <x:c r="K101" s="548" t="str">
+        <x:v>Chase pending — Sep 15</x:v>
+      </x:c>
+      <x:c r="L101" s="548" t="str">
+        <x:v>Pending list</x:v>
+      </x:c>
+      <x:c r="M101" s="548" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
     </x:row>
     <x:row r="102">
-      <x:c r="A102" s="548"/>
-      <x:c r="B102" s="478"/>
-      <x:c r="C102" s="548"/>
-      <x:c r="D102" s="547"/>
-      <x:c r="E102" s="548"/>
-      <x:c r="F102" s="548"/>
-      <x:c r="G102" s="548"/>
-      <x:c r="H102" s="574" t="str">
+      <x:c r="A102" s="548" t="str">
+        <x:v>Chase</x:v>
+      </x:c>
+      <x:c r="B102" s="478" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="C102" s="548" t="str">
+        <x:v>EXXON</x:v>
+      </x:c>
+      <x:c r="D102" s="547" t="n">
+        <x:v>39.41</x:v>
+      </x:c>
+      <x:c r="E102" s="548" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="F102" s="548" t="str">
+        <x:v>Fuel</x:v>
+      </x:c>
+      <x:c r="G102" s="548" t="str">
+        <x:v>Include</x:v>
+      </x:c>
+      <x:c r="H102" s="574" t="n">
         <x:f>IF(B102="","",B102-WEEKDAY(B102-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I102" s="548"/>
-      <x:c r="J102" s="548"/>
-      <x:c r="K102" s="548"/>
-      <x:c r="L102" s="548"/>
-      <x:c r="M102" s="548"/>
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="I102" s="548" t="str">
+        <x:v>chase-2026-09-15-exxon-3941</x:v>
+      </x:c>
+      <x:c r="J102" s="548" t="str">
+        <x:v>Pending in Sep. 15 Chase activity</x:v>
+      </x:c>
+      <x:c r="K102" s="548" t="str">
+        <x:v>Chase pending — Sep 15</x:v>
+      </x:c>
+      <x:c r="L102" s="548" t="str">
+        <x:v>Pending list</x:v>
+      </x:c>
+      <x:c r="M102" s="548" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
     </x:row>
     <x:row r="103">
-      <x:c r="A103" s="548"/>
-      <x:c r="B103" s="478"/>
-      <x:c r="C103" s="548"/>
-      <x:c r="D103" s="547"/>
-      <x:c r="E103" s="548"/>
-      <x:c r="F103" s="548"/>
-      <x:c r="G103" s="548"/>
-      <x:c r="H103" s="574" t="str">
+      <x:c r="A103" s="548" t="str">
+        <x:v>Chase</x:v>
+      </x:c>
+      <x:c r="B103" s="478" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="C103" s="548" t="str">
+        <x:v>Target</x:v>
+      </x:c>
+      <x:c r="D103" s="547" t="n">
+        <x:v>25.29</x:v>
+      </x:c>
+      <x:c r="E103" s="548" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="F103" s="548" t="str">
+        <x:v>Shopping / personal care</x:v>
+      </x:c>
+      <x:c r="G103" s="548" t="str">
+        <x:v>Include</x:v>
+      </x:c>
+      <x:c r="H103" s="574" t="n">
         <x:f>IF(B103="","",B103-WEEKDAY(B103-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I103" s="548"/>
-      <x:c r="J103" s="548"/>
-      <x:c r="K103" s="548"/>
-      <x:c r="L103" s="548"/>
-      <x:c r="M103" s="548"/>
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="I103" s="548" t="str">
+        <x:v>chase-2026-09-15-target-2529</x:v>
+      </x:c>
+      <x:c r="J103" s="548" t="str">
+        <x:v>Pending in Sep. 15 Chase activity</x:v>
+      </x:c>
+      <x:c r="K103" s="548" t="str">
+        <x:v>Chase pending — Sep 15</x:v>
+      </x:c>
+      <x:c r="L103" s="548" t="str">
+        <x:v>Pending list</x:v>
+      </x:c>
+      <x:c r="M103" s="548" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
     </x:row>
     <x:row r="104">
-      <x:c r="A104" s="548"/>
-      <x:c r="B104" s="478"/>
-      <x:c r="C104" s="548"/>
-      <x:c r="D104" s="547"/>
-      <x:c r="E104" s="548"/>
-      <x:c r="F104" s="548"/>
-      <x:c r="G104" s="548"/>
-      <x:c r="H104" s="574" t="str">
+      <x:c r="A104" s="548" t="str">
+        <x:v>Chase</x:v>
+      </x:c>
+      <x:c r="B104" s="478" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="C104" s="548" t="str">
+        <x:v>INVINCIBLE APPCHARGE</x:v>
+      </x:c>
+      <x:c r="D104" s="547" t="n">
+        <x:v>45.89</x:v>
+      </x:c>
+      <x:c r="E104" s="548" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="F104" s="548" t="str">
+        <x:v>Invincibles + other Apple</x:v>
+      </x:c>
+      <x:c r="G104" s="548" t="str">
+        <x:v>Include</x:v>
+      </x:c>
+      <x:c r="H104" s="574" t="n">
         <x:f>IF(B104="","",B104-WEEKDAY(B104-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I104" s="548"/>
-      <x:c r="J104" s="548"/>
-      <x:c r="K104" s="548"/>
-      <x:c r="L104" s="548"/>
-      <x:c r="M104" s="548"/>
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="I104" s="548" t="str">
+        <x:v>chase-2026-09-15-invincible-4589</x:v>
+      </x:c>
+      <x:c r="J104" s="548" t="str">
+        <x:v>Pending in Sep. 15 Chase activity</x:v>
+      </x:c>
+      <x:c r="K104" s="548" t="str">
+        <x:v>Chase pending — Sep 15</x:v>
+      </x:c>
+      <x:c r="L104" s="548" t="str">
+        <x:v>Pending list</x:v>
+      </x:c>
+      <x:c r="M104" s="548" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
     </x:row>
     <x:row r="105">
-      <x:c r="A105" s="548"/>
-      <x:c r="B105" s="478"/>
-      <x:c r="C105" s="548"/>
-      <x:c r="D105" s="547"/>
-      <x:c r="E105" s="548"/>
-      <x:c r="F105" s="548"/>
-      <x:c r="G105" s="548"/>
-      <x:c r="H105" s="574" t="str">
+      <x:c r="A105" s="548" t="str">
+        <x:v>Chase</x:v>
+      </x:c>
+      <x:c r="B105" s="478" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="C105" s="548" t="str">
+        <x:v>Starbucks</x:v>
+      </x:c>
+      <x:c r="D105" s="547" t="n">
+        <x:v>6.22</x:v>
+      </x:c>
+      <x:c r="E105" s="548" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="F105" s="548" t="str">
+        <x:v>Starbucks</x:v>
+      </x:c>
+      <x:c r="G105" s="548" t="str">
+        <x:v>Include</x:v>
+      </x:c>
+      <x:c r="H105" s="574" t="n">
         <x:f>IF(B105="","",B105-WEEKDAY(B105-2,1)+1)</x:f>
-      </x:c>
-      <x:c r="I105" s="548"/>
-      <x:c r="J105" s="548"/>
-      <x:c r="K105" s="548"/>
-      <x:c r="L105" s="548"/>
-      <x:c r="M105" s="548"/>
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="I105" s="548" t="str">
+        <x:v>chase-2026-09-15-starbucks-622</x:v>
+      </x:c>
+      <x:c r="J105" s="548" t="str">
+        <x:v>Pending in Sep. 15 Chase activity</x:v>
+      </x:c>
+      <x:c r="K105" s="548" t="str">
+        <x:v>Chase pending — Sep 15</x:v>
+      </x:c>
+      <x:c r="L105" s="548" t="str">
+        <x:v>Pending list</x:v>
+      </x:c>
+      <x:c r="M105" s="548" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="548"/>
@@ -16441,11 +17030,11 @@
       </x:c>
       <x:c r="D20" s="459" t="n">
         <x:f>'Support - Promo Detail'!F12</x:f>
-        <x:v>148.616</x:v>
+        <x:v>148.615</x:v>
       </x:c>
       <x:c r="E20" s="480" t="n">
         <x:f>D20</x:f>
-        <x:v>148.616</x:v>
+        <x:v>148.615</x:v>
       </x:c>
       <x:c r="F20" s="423" t="str">
         <x:v>Formula linked below</x:v>
@@ -16694,7 +17283,7 @@
       <x:c r="D32" s="482"/>
       <x:c r="E32" s="482" t="n">
         <x:f>SUM(E12:E31)</x:f>
-        <x:v>1531.6146692307693</x:v>
+        <x:v>1531.6136692307691</x:v>
       </x:c>
       <x:c r="F32" s="481"/>
     </x:row>
@@ -16715,7 +17304,7 @@
       <x:c r="D34" s="501"/>
       <x:c r="E34" s="501" t="n">
         <x:f>D8-E32</x:f>
-        <x:v>-188.24466923076943</x:v>
+        <x:v>-188.24366923076923</x:v>
       </x:c>
       <x:c r="F34" s="503"/>
     </x:row>
@@ -16787,7 +17376,7 @@
       <x:c r="B41" s="423"/>
       <x:c r="C41" s="480" t="n">
         <x:f>E32</x:f>
-        <x:v>1531.6146692307693</x:v>
+        <x:v>1531.6136692307691</x:v>
       </x:c>
       <x:c r="D41" s="423"/>
       <x:c r="E41" s="423"/>
@@ -16949,7 +17538,7 @@
       </x:c>
       <x:c r="C7" s="459" t="n">
         <x:f>'Support - Budget Inputs'!E20</x:f>
-        <x:v>148.616</x:v>
+        <x:v>148.615</x:v>
       </x:c>
       <x:c r="D7" s="478" t="n">
         <x:v>46305</x:v>

</xml_diff>

<commit_message>
Record zero Prime and Discover balances
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R0d58d46c8b0c4216"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R6bdf36e212a84f60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R3d5cdcab761248ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="Rd9b62d36e14a490d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="Rabbfabd2f0114dbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="Rfb86f398aff24cc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R2b236d01cb8946b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R7b222af8d7e44e89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="Rfd7788d394c74dff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R3fc0106e3fb040b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R3079e3517b414031"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R300128cabed1444a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R5e5c740167cb400b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="Raf532aa1deb34965"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="Rf1bb359141a74d34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R8ba5e0cac0ea45f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R03b2dc6223ff4b5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R2a7f2e1dc1a344a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R4f63c185ff424bcf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R0972638c21e343a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R9da1fa26e3c04dfd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R55862b8dd89f45f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R4c53f45aab4a46b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R48cb6c1040ff440a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="Rb448ec3b14bf4993"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R8ed3867eb2d443f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R7ae30cdbfef94d49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R61f2f7e7f76d4bf1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R9b2626a744964e90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="Ra91f42feb1c449ce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3360,10 +3360,10 @@
         <x:v>Discover card</x:v>
       </x:c>
       <x:c r="B7" s="547" t="n">
-        <x:v>48.27</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C7" s="547" t="n">
-        <x:v>48.27</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D7" s="478"/>
       <x:c r="E7" s="423" t="str">
@@ -3373,7 +3373,7 @@
         <x:v>USD</x:v>
       </x:c>
       <x:c r="G7" s="423" t="str">
-        <x:v>User-confirmed carried-forward amount to pay. Latest screenshot showed Nationwide Pet $48.27 pending; verify it has posted before submitting payment.</x:v>
+        <x:v>User-reported current balance $0.00 on Sep. 15; activity was not captured, so any new charges still need review.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -3415,7 +3415,7 @@
         <x:v>USD</x:v>
       </x:c>
       <x:c r="G9" s="423" t="str">
-        <x:v>Current balance $0 in Sep. 9 app screenshot; no payment due</x:v>
+        <x:v>User-reported current balance $0.00 on Sep. 15; activity was not captured, so any new charges still need review.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -4211,7 +4211,7 @@
         <x:v>Needed</x:v>
       </x:c>
       <x:c r="J17" s="423" t="str">
-        <x:v>Capture current balance and any activity</x:v>
+        <x:v>Balance confirmed $0.00; capture activity before verification</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="30" customHeight="1">
@@ -4240,7 +4240,7 @@
         <x:v>Needed</x:v>
       </x:c>
       <x:c r="J18" s="423" t="str">
-        <x:v>Capture current balance and activity</x:v>
+        <x:v>Balance confirmed $0.00; capture activity before verification</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="30" customHeight="1">
@@ -5605,7 +5605,7 @@
       </x:c>
       <x:c r="C6" s="458" t="str">
         <x:f>COUNTIFS(F9:F21,"Manual",E9:E21,"☑ Done")&amp;" / "&amp;COUNTIF(F9:F21,"Manual")&amp;" manual payments complete"</x:f>
-        <x:v>5 / 7 manual payments complete</x:v>
+        <x:v>5 / 5 manual payments complete</x:v>
       </x:c>
       <x:c r="D6" s="458" t="str">
         <x:v>Await remaining imports</x:v>
@@ -5700,19 +5700,19 @@
         <x:v>Discover card</x:v>
       </x:c>
       <x:c r="C11" s="423" t="str">
-        <x:v>$48.27 carried-forward balance to pay</x:v>
+        <x:v>Current balance $0.00</x:v>
       </x:c>
       <x:c r="D11" s="468" t="n">
-        <x:v>48.27</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E11" s="460" t="str">
-        <x:v>☐ Pay now</x:v>
+        <x:v>— Not due</x:v>
       </x:c>
       <x:c r="F11" s="461" t="str">
-        <x:v>Manual</x:v>
+        <x:v>Not due</x:v>
       </x:c>
       <x:c r="G11" s="423" t="str">
-        <x:v>User-confirmed amount owed; latest screenshot showed this charge pending, so confirm it can be paid before submitting</x:v>
+        <x:v>No payment needed; activity still needs capture</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="28" customHeight="1">
@@ -5723,7 +5723,7 @@
         <x:v>Prime Visa</x:v>
       </x:c>
       <x:c r="C12" s="423" t="str">
-        <x:v>No balance due</x:v>
+        <x:v>Current balance $0.00</x:v>
       </x:c>
       <x:c r="D12" s="468" t="n">
         <x:v>0</x:v>
@@ -5735,7 +5735,7 @@
         <x:v>Not due</x:v>
       </x:c>
       <x:c r="G12" s="423" t="str">
-        <x:v>No payment needed</x:v>
+        <x:v>No payment needed; activity still needs capture</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="28" customHeight="1">
@@ -5936,17 +5936,17 @@
       </x:c>
       <x:c r="D21" s="468" t="n">
         <x:f>MAX(0,E23+E25-E24)</x:f>
-        <x:v>48.269000000000005</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E21" s="460" t="str">
-        <x:v>☐ Pay now</x:v>
+        <x:v>— Not needed</x:v>
       </x:c>
       <x:c r="F21" s="461" t="str">
-        <x:v>Manual</x:v>
+        <x:v>Not needed</x:v>
       </x:c>
       <x:c r="G21" s="423" t="str">
         <x:f>IF(D21=0,"No transfer needed after net rent funding","Additional funding required after adding Discover")</x:f>
-        <x:v>Additional funding required after adding Discover</x:v>
+        <x:v>No transfer needed after net rent funding</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -5957,7 +5957,7 @@
       <x:c r="C22" s="458"/>
       <x:c r="D22" s="462" t="n">
         <x:f>SUM(D9:D16,D18:D20)</x:f>
-        <x:v>1275.049</x:v>
+        <x:v>1226.779</x:v>
       </x:c>
       <x:c r="E22" s="423"/>
       <x:c r="F22" s="423"/>
@@ -5972,7 +5972,7 @@
       <x:c r="D23" s="463"/>
       <x:c r="E23" s="469" t="n">
         <x:f>SUM(D9:D16,D18:D20)</x:f>
-        <x:v>1275.049</x:v>
+        <x:v>1226.779</x:v>
       </x:c>
       <x:c r="F23" s="423"/>
       <x:c r="G23" s="423"/>
@@ -6012,7 +6012,7 @@
       <x:c r="D26" s="463"/>
       <x:c r="E26" s="471" t="n">
         <x:f>D21</x:f>
-        <x:v>48.269000000000005</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F26" s="423"/>
       <x:c r="G26" s="423"/>

</xml_diff>

<commit_message>
Update personal safe cash balance
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R7f09ea6ccd294842"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="Raf341bb9f785406b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R080343ac94f4470f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="Re736f880a0d84b1a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R9db3daf16ed64cbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R2a81ecedfff54c52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R7c48e14e04684783"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="Rcbe53dc011e04161"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R986e533646f04176"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R0a0a4fd1ed0a493a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R51f7bc557b024cfc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="Rdabc2c91374e4216"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R2cf7ba78fb1a4de3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="Racb49b4577334b48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R39db33197fb34a83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R7f0d213f44634d5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R1f3acb4914ea4721"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R57581d20bd044359"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R44e84e52a7c84c56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R627ef7dd3c4f42d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="Re460ec84b1e243c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R2a0368fc4f124532"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="Re18a7a56606d43a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R3dd3bad0d8984d66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R298bddae0541406a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="Rfe703a9586c14d05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R08857d9f5fbf4419"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R8b809d0f8f494ba8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R86aa40cbbfbf4907"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R4f6ebb0941174dc6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3906,13 +3906,13 @@
     </x:row>
     <x:row r="7" ht="45" customHeight="1">
       <x:c r="A7" s="467" t="n">
-        <x:v>46274</x:v>
+        <x:v>46280</x:v>
       </x:c>
       <x:c r="B7" s="415" t="str">
         <x:v>Personal safe cash</x:v>
       </x:c>
       <x:c r="C7" s="468" t="n">
-        <x:v>220</x:v>
+        <x:v>510</x:v>
       </x:c>
       <x:c r="D7" s="468" t="n">
         <x:v>0</x:v>
@@ -3921,10 +3921,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F7" s="468" t="n">
-        <x:v>220</x:v>
+        <x:v>510</x:v>
       </x:c>
       <x:c r="G7" s="415" t="str">
-        <x:v>Wife’s Sep. 9 income held as cash; $160 added to the prior $60. Excluded from Wells/Wealthfront funding.</x:v>
+        <x:v>Current user-reported personal-safe cash balance. Savings-only and excluded from Wells/Wealthfront funding and spending-capacity calculations.</x:v>
       </x:c>
       <x:c r="H7" s="563"/>
       <x:c r="I7" s="563"/>
@@ -7060,7 +7060,7 @@
       </x:c>
       <x:c r="B26" s="498" t="n">
         <x:f>'Support - Account Snapshots'!F7</x:f>
-        <x:v>220</x:v>
+        <x:v>510</x:v>
       </x:c>
       <x:c r="C26" s="454"/>
       <x:c r="D26" s="454"/>
@@ -7319,7 +7319,7 @@
       </x:c>
       <x:c r="B6" s="553" t="n">
         <x:f>'Support - Account Snapshots'!F7</x:f>
-        <x:v>220</x:v>
+        <x:v>510</x:v>
       </x:c>
       <x:c r="C6" s="530" t="str">
         <x:v>Rent due estimate</x:v>
@@ -7337,7 +7337,7 @@
       </x:c>
       <x:c r="B7" s="554" t="n">
         <x:f>SUM(B5:B6)</x:f>
-        <x:v>12246.13</x:v>
+        <x:v>12536.13</x:v>
       </x:c>
       <x:c r="C7" s="530" t="str">
         <x:v>Tagged rent reserve</x:v>
@@ -7373,7 +7373,7 @@
       </x:c>
       <x:c r="B9" s="556" t="n">
         <x:f>B7-B8</x:f>
-        <x:v>260.17229999999654</x:v>
+        <x:v>550.1722999999965</x:v>
       </x:c>
       <x:c r="C9" s="535" t="str">
         <x:v>Confirmed funding vs. monthly plan</x:v>
@@ -16767,7 +16767,7 @@
       </x:c>
       <x:c r="C7" s="447" t="n">
         <x:f>'Support - Account Snapshots'!F7</x:f>
-        <x:v>220</x:v>
+        <x:v>510</x:v>
       </x:c>
       <x:c r="D7" s="447" t="n">
         <x:v>0</x:v>

</xml_diff>

<commit_message>
Rebuild Sep 15 Tuesday payment plan
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R7f0d213f44634d5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R1f3acb4914ea4721"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R57581d20bd044359"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R44e84e52a7c84c56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R627ef7dd3c4f42d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="Re460ec84b1e243c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R2a0368fc4f124532"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="Re18a7a56606d43a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R3dd3bad0d8984d66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R298bddae0541406a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="Rfe703a9586c14d05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R08857d9f5fbf4419"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R8b809d0f8f494ba8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R86aa40cbbfbf4907"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R4f6ebb0941174dc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R9a274b19d89a4f8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R6d205fb3cdf4401a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R60fdee5762274671"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R29027ba59ecd466b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R9b0f93b58f5b4171"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="Red531464ff2a4f6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="Ra9ece658ef484504"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R94362913de684361"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R9d2c695432b0427f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R4ab4bc48fd87447e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="Rc423bd8474694a5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R9bb0e29e97ab4409"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R956fea06646b4a01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R4e812e6f22b34b5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="Rc678d3ce5ebe448e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2942,10 +2942,10 @@
         <x:v>Cash plan</x:v>
       </x:c>
       <x:c r="B7" s="434" t="str">
-        <x:v>Ready</x:v>
+        <x:v>Built</x:v>
       </x:c>
       <x:c r="C7" s="425" t="str">
-        <x:v>All current required source checkpoints are verified</x:v>
+        <x:v>Tuesday Review reflects all verified current actions</x:v>
       </x:c>
       <x:c r="D7" s="415"/>
       <x:c r="E7" s="397" t="str">
@@ -2967,10 +2967,10 @@
         <x:v>Next action</x:v>
       </x:c>
       <x:c r="B8" s="435" t="str">
-        <x:v>Build plan</x:v>
+        <x:v>Execute plan</x:v>
       </x:c>
       <x:c r="C8" s="428" t="str">
-        <x:v>Rebuild Tuesday Review from this week’s verified actions</x:v>
+        <x:v>Use Tuesday Review checkoffs while you pay or transfer funds</x:v>
       </x:c>
       <x:c r="D8" s="415"/>
       <x:c r="E8" s="397" t="str">
@@ -5577,14 +5577,14 @@
         <x:v>8 of 8 source sets verified</x:v>
       </x:c>
       <x:c r="B6" s="446" t="str">
-        <x:v>Sep 1–Sep 7 purchases</x:v>
+        <x:v>Sep 8–Sep 14 purchases</x:v>
       </x:c>
       <x:c r="C6" s="446" t="str">
         <x:f>COUNTIFS(F9:F21,"Manual",E9:E21,"☑ Done")&amp;" / "&amp;COUNTIF(F9:F21,"Manual")&amp;" manual payments complete"</x:f>
-        <x:v>5 / 5 manual payments complete</x:v>
+        <x:v>0 / 5 manual payments complete</x:v>
       </x:c>
       <x:c r="D6" s="446" t="str">
-        <x:v>Ready to rebuild</x:v>
+        <x:v>Current plan — Sep 15</x:v>
       </x:c>
       <x:c r="E6" s="446"/>
       <x:c r="F6" s="446"/>
@@ -5630,19 +5630,19 @@
         <x:v>Chase Sapphire</x:v>
       </x:c>
       <x:c r="C9" s="415" t="str">
-        <x:v>Current Sep. 9 balance</x:v>
+        <x:v>Current Sep. 15 balance</x:v>
       </x:c>
       <x:c r="D9" s="456" t="n">
-        <x:v>266.96</x:v>
+        <x:v>786.38</x:v>
       </x:c>
       <x:c r="E9" s="448" t="str">
-        <x:v>☑ Done</x:v>
+        <x:v>☐ Pay now</x:v>
       </x:c>
       <x:c r="F9" s="449" t="str">
         <x:v>Manual</x:v>
       </x:c>
       <x:c r="G9" s="415" t="str">
-        <x:v>Pay the current balance if maintaining the weekly payoff routine</x:v>
+        <x:v>Pay the current balance, including listed pending charges</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="28" customHeight="1">
@@ -5653,19 +5653,19 @@
         <x:v>Citi card</x:v>
       </x:c>
       <x:c r="C10" s="415" t="str">
-        <x:v>Current Sep. 9 balance</x:v>
+        <x:v>Current Sep. 15 balance</x:v>
       </x:c>
       <x:c r="D10" s="456" t="n">
-        <x:v>132.09</x:v>
+        <x:v>106.26</x:v>
       </x:c>
       <x:c r="E10" s="448" t="str">
-        <x:v>☑ Done</x:v>
+        <x:v>☐ Pay now</x:v>
       </x:c>
       <x:c r="F10" s="449" t="str">
         <x:v>Manual</x:v>
       </x:c>
       <x:c r="G10" s="415" t="str">
-        <x:v>Pay the current balance if maintaining the weekly payoff routine</x:v>
+        <x:v>Pay the current balance, including listed pending charges</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="28" customHeight="1">
@@ -5752,13 +5752,13 @@
         <x:v>148.615</x:v>
       </x:c>
       <x:c r="E14" s="448" t="str">
-        <x:v>☑ Done</x:v>
+        <x:v>☐ Pay now</x:v>
       </x:c>
       <x:c r="F14" s="449" t="str">
         <x:v>Manual</x:v>
       </x:c>
       <x:c r="G14" s="415" t="str">
-        <x:v>Five weekly payments remain before Oct. 10</x:v>
+        <x:v>Four weekly payments remain before Oct. 10</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="28" customHeight="1">
@@ -5769,19 +5769,20 @@
         <x:v>Rent fund — October</x:v>
       </x:c>
       <x:c r="C15" s="415" t="str">
-        <x:v>Actual Sep. 9 funding retained</x:v>
+        <x:v>Only verified Wells capacity after required actions</x:v>
       </x:c>
       <x:c r="D15" s="456" t="n">
-        <x:v>178.49169230769235</x:v>
+        <x:f>MAX(0,E24-SUM(D9:D14,D16:D20)-E25)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E15" s="448" t="str">
-        <x:v>☑ Done</x:v>
+        <x:v>— Not needed</x:v>
       </x:c>
       <x:c r="F15" s="449" t="str">
-        <x:v>Manual</x:v>
+        <x:v>Not needed</x:v>
       </x:c>
       <x:c r="G15" s="415" t="str">
-        <x:v>Actual Sep. 9 transfer retained; do not revise this completed funding amount</x:v>
+        <x:v>No rent contribution this Tuesday because required actions exceed Wells cash</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="28" customHeight="1">
@@ -5799,7 +5800,7 @@
         <x:v>172.26230769230767</x:v>
       </x:c>
       <x:c r="E16" s="448" t="str">
-        <x:v>☑ Done</x:v>
+        <x:v>☐ Pay now</x:v>
       </x:c>
       <x:c r="F16" s="449" t="str">
         <x:v>Manual</x:v>
@@ -5816,7 +5817,7 @@
         <x:v>Fidelity Roth IRA</x:v>
       </x:c>
       <x:c r="C17" s="415" t="str">
-        <x:v>Pending; already in Wells available balance</x:v>
+        <x:v>Weekly automatic transfer</x:v>
       </x:c>
       <x:c r="D17" s="456" t="n">
         <x:v>75</x:v>
@@ -5828,7 +5829,7 @@
         <x:v>Automatic</x:v>
       </x:c>
       <x:c r="G17" s="415" t="str">
-        <x:v>Do not count again in cash required</x:v>
+        <x:v>Automatic commitment; included in cash required</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="28" customHeight="1">
@@ -5839,7 +5840,7 @@
         <x:v>PayPal cruise savings</x:v>
       </x:c>
       <x:c r="C18" s="415" t="str">
-        <x:v>Flexible savings contribution</x:v>
+        <x:v>Weekly automatic transfer</x:v>
       </x:c>
       <x:c r="D18" s="456" t="n">
         <x:v>85</x:v>
@@ -5862,7 +5863,7 @@
         <x:v>PayPal tuition savings</x:v>
       </x:c>
       <x:c r="C19" s="415" t="str">
-        <x:v>Weekly scheduled transfer</x:v>
+        <x:v>Weekly automatic transfer</x:v>
       </x:c>
       <x:c r="D19" s="456" t="n">
         <x:v>193.36</x:v>
@@ -5885,7 +5886,7 @@
         <x:v>PayPal future-expenses savings</x:v>
       </x:c>
       <x:c r="C20" s="415" t="str">
-        <x:v>Flexible savings contribution</x:v>
+        <x:v>Weekly automatic transfer</x:v>
       </x:c>
       <x:c r="D20" s="456" t="n">
         <x:v>50</x:v>
@@ -5908,21 +5909,21 @@
         <x:v>Wealthfront to Wells</x:v>
       </x:c>
       <x:c r="C21" s="415" t="str">
-        <x:v>Cover a remaining cash shortfall</x:v>
+        <x:v>Cover the verified cash shortfall and leave $1 in Wells</x:v>
       </x:c>
       <x:c r="D21" s="456" t="n">
         <x:f>MAX(0,E23+E25-E24)</x:f>
-        <x:v>0</x:v>
+        <x:v>225.157307692308</x:v>
       </x:c>
       <x:c r="E21" s="448" t="str">
-        <x:v>— Not needed</x:v>
+        <x:v>☐ Pay now</x:v>
       </x:c>
       <x:c r="F21" s="449" t="str">
-        <x:v>Not needed</x:v>
+        <x:v>Manual</x:v>
       </x:c>
       <x:c r="G21" s="415" t="str">
-        <x:f>IF(D21=0,"No transfer needed after net rent funding","Additional funding required after adding Discover")</x:f>
-        <x:v>No transfer needed after net rent funding</x:v>
+        <x:f>IF(D21=0,"No transfer needed; leave $1 in Wells","Transfer this amount from Wealthfront to leave $1 in Wells")</x:f>
+        <x:v>Transfer this amount from Wealthfront to leave $1 in Wells</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -5932,8 +5933,8 @@
       <x:c r="B22" s="446"/>
       <x:c r="C22" s="446"/>
       <x:c r="D22" s="450" t="n">
-        <x:f>SUM(D9:D16,D18:D20)</x:f>
-        <x:v>1226.779</x:v>
+        <x:f>SUM(D9:D20)</x:f>
+        <x:v>1616.877307692308</x:v>
       </x:c>
       <x:c r="E22" s="415"/>
       <x:c r="F22" s="415"/>
@@ -5947,21 +5948,22 @@
       <x:c r="C23" s="451"/>
       <x:c r="D23" s="451"/>
       <x:c r="E23" s="457" t="n">
-        <x:f>SUM(D9:D16,D18:D20)</x:f>
-        <x:v>1226.779</x:v>
+        <x:f>SUM(D9:D20)</x:f>
+        <x:v>1616.877307692308</x:v>
       </x:c>
       <x:c r="F23" s="415"/>
       <x:c r="G23" s="415"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="451" t="str">
-        <x:v>Wells available now after pending Fidelity</x:v>
+        <x:v>Wells available from verified import</x:v>
       </x:c>
       <x:c r="B24" s="451"/>
       <x:c r="C24" s="451"/>
       <x:c r="D24" s="451"/>
       <x:c r="E24" s="458" t="n">
-        <x:v>1227.78</x:v>
+        <x:f>'1. Start'!B5</x:f>
+        <x:v>1392.72</x:v>
       </x:c>
       <x:c r="F24" s="415"/>
       <x:c r="G24" s="415"/>
@@ -5988,7 +5990,7 @@
       <x:c r="D26" s="451"/>
       <x:c r="E26" s="459" t="n">
         <x:f>D21</x:f>
-        <x:v>0</x:v>
+        <x:v>225.157307692308</x:v>
       </x:c>
       <x:c r="F26" s="415"/>
       <x:c r="G26" s="415"/>
@@ -7344,7 +7346,7 @@
       </x:c>
       <x:c r="D7" s="553" t="n">
         <x:f>B39</x:f>
-        <x:v>178.49169230769235</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E7" s="415"/>
       <x:c r="F7" s="415"/>
@@ -7362,7 +7364,7 @@
       </x:c>
       <x:c r="D8" s="553" t="n">
         <x:f>E36</x:f>
-        <x:v>1021.5083076923077</x:v>
+        <x:v>1200</x:v>
       </x:c>
       <x:c r="E8" s="415"/>
       <x:c r="F8" s="415"/>
@@ -7380,7 +7382,7 @@
       </x:c>
       <x:c r="D9" s="556" t="n">
         <x:f>E34</x:f>
-        <x:v>-1021.5083076923077</x:v>
+        <x:v>-1200</x:v>
       </x:c>
       <x:c r="E9" s="415"/>
       <x:c r="F9" s="415"/>
@@ -7610,11 +7612,11 @@
       </x:c>
       <x:c r="C26" s="418" t="n">
         <x:f>'2. Tuesday Review'!D15</x:f>
-        <x:v>178.49169230769235</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D26" s="543" t="n">
         <x:f>C26-B26</x:f>
-        <x:v>-121.50830769230765</x:v>
+        <x:v>-300</x:v>
       </x:c>
       <x:c r="E26" s="395" t="str">
         <x:v>Wells cash capacity</x:v>
@@ -7693,11 +7695,11 @@
       </x:c>
       <x:c r="C30" s="540" t="n">
         <x:f>SUM(C26:C29)</x:f>
-        <x:v>178.49169230769235</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D30" s="540" t="n">
         <x:f>C30-B30</x:f>
-        <x:v>-1021.5083076923077</x:v>
+        <x:v>-1200</x:v>
       </x:c>
       <x:c r="E30" s="539"/>
       <x:c r="F30" s="539"/>
@@ -7741,7 +7743,7 @@
       </x:c>
       <x:c r="E34" s="527" t="n">
         <x:f>D30</x:f>
-        <x:v>-1021.5083076923077</x:v>
+        <x:v>-1200</x:v>
       </x:c>
       <x:c r="F34" s="415"/>
     </x:row>
@@ -7758,7 +7760,7 @@
       </x:c>
       <x:c r="E35" s="531" t="n">
         <x:f>MAX(0,$B$38-$B$39)</x:f>
-        <x:v>1021.5083076923077</x:v>
+        <x:v>1200</x:v>
       </x:c>
       <x:c r="F35" s="415"/>
     </x:row>
@@ -7775,7 +7777,7 @@
       </x:c>
       <x:c r="E36" s="531" t="n">
         <x:f>E35</x:f>
-        <x:v>1021.5083076923077</x:v>
+        <x:v>1200</x:v>
       </x:c>
       <x:c r="F36" s="415"/>
     </x:row>
@@ -7820,7 +7822,7 @@
       </x:c>
       <x:c r="B39" s="536" t="n">
         <x:f>B36+C30+B37</x:f>
-        <x:v>178.49169230769235</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C39" s="415"/>
       <x:c r="D39" s="516" t="str">
@@ -8088,10 +8090,18 @@
         <x:f>A7-1</x:f>
         <x:v>46279</x:v>
       </x:c>
-      <x:c r="D7" s="537"/>
-      <x:c r="E7" s="537"/>
-      <x:c r="F7" s="537"/>
-      <x:c r="G7" s="538"/>
+      <x:c r="D7" s="537" t="n">
+        <x:v>1392.72</x:v>
+      </x:c>
+      <x:c r="E7" s="537" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F7" s="537" t="n">
+        <x:v>1616.8773076923076</x:v>
+      </x:c>
+      <x:c r="G7" s="538" t="str">
+        <x:v>Plan created — Sep 15</x:v>
+      </x:c>
       <x:c r="H7" s="537"/>
       <x:c r="I7" s="468" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$H$5:$H$304,B7,'Support - Ledger'!$E$5:$E$304,"Posted",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
@@ -8108,7 +8118,9 @@
       <x:c r="L7" s="468" t="str">
         <x:f>IF(H7="","",H7-K7)</x:f>
       </x:c>
-      <x:c r="M7" s="538"/>
+      <x:c r="M7" s="538" t="str">
+        <x:v>Sep. 15 payment plan built from verified imports. It uses a $225.16 general cash top-up from Wealthfront and makes no rent contribution this Tuesday.</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="22" customHeight="1">
       <x:c r="A8" s="467" t="n">
@@ -8904,7 +8916,7 @@
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="G5:G30">
-      <x:formula1>"In progress,Plan created — Sep 9,Data verified — Sep 9,Legacy — not source-audited,✓ Completed,Needs review"</x:formula1>
+      <x:formula1>"In progress,Plan created — Sep 9,Plan created — Sep 15,Data verified — Sep 9,Legacy — not source-audited,✓ Completed,Needs review"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -17460,7 +17472,7 @@
       </x:c>
       <x:c r="C5" s="447" t="n">
         <x:f>'2. Tuesday Review'!D15</x:f>
-        <x:v>178.49169230769235</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D5" s="466" t="n">
         <x:v>46296</x:v>

</xml_diff>

<commit_message>
Record September rent fund contribution
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R9a274b19d89a4f8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R6d205fb3cdf4401a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R60fdee5762274671"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R29027ba59ecd466b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R9b0f93b58f5b4171"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="Red531464ff2a4f6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="Ra9ece658ef484504"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R94362913de684361"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R9d2c695432b0427f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R4ab4bc48fd87447e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="Rc423bd8474694a5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R9bb0e29e97ab4409"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R956fea06646b4a01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R4e812e6f22b34b5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="Rc678d3ce5ebe448e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R9ccd4b59498940ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="Rd0ac719bc0d54a33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R26f2b1132efa4b16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R3ad549b54a784fb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R426df1a8c3db4a2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="Rb1a807762f35430a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="Re587bc169cef418f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R90d4ea5846264bc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R9c15e4fe657b4992"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R879c71dbc3e54039"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="Rbfd11d7cd4124d77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R5baa4910206b4c78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="Rda76e86900d3449f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R93b26231d4e645a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R4db638e8af5c4dff"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7346,7 +7346,7 @@
       </x:c>
       <x:c r="D7" s="553" t="n">
         <x:f>B39</x:f>
-        <x:v>0</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="E7" s="415"/>
       <x:c r="F7" s="415"/>
@@ -7364,7 +7364,7 @@
       </x:c>
       <x:c r="D8" s="553" t="n">
         <x:f>E36</x:f>
-        <x:v>1200</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="E8" s="415"/>
       <x:c r="F8" s="415"/>
@@ -7382,7 +7382,7 @@
       </x:c>
       <x:c r="D9" s="556" t="n">
         <x:f>E34</x:f>
-        <x:v>-1200</x:v>
+        <x:v>-900</x:v>
       </x:c>
       <x:c r="E9" s="415"/>
       <x:c r="F9" s="415"/>
@@ -7611,18 +7611,17 @@
         <x:v>300</x:v>
       </x:c>
       <x:c r="C26" s="418" t="n">
-        <x:f>'2. Tuesday Review'!D15</x:f>
-        <x:v>0</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="D26" s="543" t="n">
         <x:f>C26-B26</x:f>
-        <x:v>-300</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E26" s="395" t="str">
-        <x:v>Wells cash capacity</x:v>
+        <x:v>Wells rent fund</x:v>
       </x:c>
       <x:c r="F26" s="419" t="str">
-        <x:v>Calculated from verified Tuesday plan</x:v>
+        <x:v>Actual Sep. 9 contribution; do not net against separate cash movements</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="25" customHeight="1">
@@ -7633,16 +7632,19 @@
         <x:f>'Support - Budget Inputs'!$E$12</x:f>
         <x:v>300</x:v>
       </x:c>
-      <x:c r="C27" s="546"/>
+      <x:c r="C27" s="546" t="n">
+        <x:f>'2. Tuesday Review'!D15</x:f>
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="D27" s="545" t="n">
         <x:f>C27-B27</x:f>
         <x:v>-300</x:v>
       </x:c>
       <x:c r="E27" s="398" t="str">
-        <x:v>Enter after review</x:v>
+        <x:v>Wells cash capacity</x:v>
       </x:c>
       <x:c r="F27" s="399" t="str">
-        <x:v>No catch-up assumed</x:v>
+        <x:v>Calculated from verified Tuesday plan</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="25" customHeight="1">
@@ -7695,11 +7697,11 @@
       </x:c>
       <x:c r="C30" s="540" t="n">
         <x:f>SUM(C26:C29)</x:f>
-        <x:v>0</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="D30" s="540" t="n">
         <x:f>C30-B30</x:f>
-        <x:v>-1200</x:v>
+        <x:v>-900</x:v>
       </x:c>
       <x:c r="E30" s="539"/>
       <x:c r="F30" s="539"/>
@@ -7743,7 +7745,7 @@
       </x:c>
       <x:c r="E34" s="527" t="n">
         <x:f>D30</x:f>
-        <x:v>-1200</x:v>
+        <x:v>-900</x:v>
       </x:c>
       <x:c r="F34" s="415"/>
     </x:row>
@@ -7760,7 +7762,7 @@
       </x:c>
       <x:c r="E35" s="531" t="n">
         <x:f>MAX(0,$B$38-$B$39)</x:f>
-        <x:v>1200</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="F35" s="415"/>
     </x:row>
@@ -7777,7 +7779,7 @@
       </x:c>
       <x:c r="E36" s="531" t="n">
         <x:f>E35</x:f>
-        <x:v>1200</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="F36" s="415"/>
     </x:row>
@@ -7822,7 +7824,7 @@
       </x:c>
       <x:c r="B39" s="536" t="n">
         <x:f>B36+C30+B37</x:f>
-        <x:v>0</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="C39" s="415"/>
       <x:c r="D39" s="516" t="str">
@@ -8047,10 +8049,10 @@
         <x:v>1227.78</x:v>
       </x:c>
       <x:c r="E6" s="468" t="n">
-        <x:v>0</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="F6" s="468" t="n">
-        <x:v>1226.78</x:v>
+        <x:v>1348.2883076923076</x:v>
       </x:c>
       <x:c r="G6" s="538" t="str">
         <x:v>✓ Completed</x:v>
@@ -8075,7 +8077,7 @@
         <x:v>26.17076923076928</x:v>
       </x:c>
       <x:c r="M6" s="538" t="str">
-        <x:v>Sep. 15 Wells capture confirmed all Sep. 9 manual actions. The $300.00 rent transfer and $121.51 Wealthfront return net to the planned $178.49 rent funding.</x:v>
+        <x:v>Sep. 15 Wells capture confirmed all Sep. 9 manual actions. $300.00 was transferred to the rent fund. The separate $121.51 Wealthfront return is not netted against rent funding.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="22" customHeight="1">
@@ -17893,19 +17895,19 @@
         <x:v>Rent fund — next month</x:v>
       </x:c>
       <x:c r="C23" s="415" t="str">
-        <x:v>Rent-payment Tuesday</x:v>
+        <x:v>Actual Sep. 9 rent funding</x:v>
       </x:c>
       <x:c r="D23" s="468" t="n">
-        <x:v>0</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="E23" s="468" t="n">
-        <x:v>0</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="F23" s="415" t="str">
         <x:v>✓ Done</x:v>
       </x:c>
       <x:c r="G23" s="415" t="str">
-        <x:v>No deposit on rent-payment Tuesday</x:v>
+        <x:v>Transferred from Wells Sep. 9</x:v>
       </x:c>
       <x:c r="H23" s="415"/>
     </x:row>

</xml_diff>

<commit_message>
Clarify Tuesday status dropdown guidance
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R4ac0db5d32304125"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R0fed117542644eca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R7b25bd767dc34862"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="Rbc7bd2b9c4284120"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R5e8d8a71794b4625"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="Rd42db0efc2294f53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R2a5b002682394d1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="Ra543e03072ce4e04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R20d09a6b47454c49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="Re14e2ac135f349a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="Rb1c5d375f1dd457e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R98d3936684134e75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="Rc761013148d7453e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="Rc9e56b5b079742a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R47ed527bf50f48e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R089fee4c43fa4af0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R86776ca9152041ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R5e160fcd6d254cc2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="Ra1570219365340ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R8095c75625f24599"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R7474bb3b666e45ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R931b4b74568d44be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R4b76625ea1734c52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R2f29b2499a5b48df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R52554885311e4634"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="Rbccc0a9b37b1450c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R1dbd7c0a037149d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R19d43b6d996d4a8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R437d1f69e3264460"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="Reabe8b1408054a8d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5516,7 +5516,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="434" t="str">
-        <x:v>Use this checklist after Start is verified. For a manual action, change the empty box to a checked box when complete. Automatic and not-due rows need no action.</x:v>
+        <x:v>Use this checklist after Start is verified. For a manual action, use the small dropdown to select ☑ when complete. Automatic and not-due rows need no action.</x:v>
       </x:c>
       <x:c r="B2" s="434"/>
       <x:c r="C2" s="434"/>
@@ -5604,7 +5604,7 @@
         <x:v>Planned amount</x:v>
       </x:c>
       <x:c r="E8" s="425" t="str">
-        <x:v>Done?</x:v>
+        <x:v>Status</x:v>
       </x:c>
       <x:c r="F8" s="425" t="str">
         <x:v>Action</x:v>

</xml_diff>

<commit_message>
Make Tuesday review preview-only
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R089fee4c43fa4af0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R86776ca9152041ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R5e160fcd6d254cc2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="Ra1570219365340ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R8095c75625f24599"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R7474bb3b666e45ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R931b4b74568d44be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R4b76625ea1734c52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R2f29b2499a5b48df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R52554885311e4634"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="Rbccc0a9b37b1450c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R1dbd7c0a037149d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R19d43b6d996d4a8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R437d1f69e3264460"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="Reabe8b1408054a8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R4f0b57e93c1747d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R875bfa1073d14b5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R8b4037e1d2564583"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R96e6caae1d364830"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R003a1fac39e342a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="Ra5a7789e1a9a4af1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="Rb2a2fa770e0f4dc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R57ee9fe374894332"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="Rc8512f0c80a04a57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R053ab9e7d4b94bf2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R3876ceb680ec423b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R43844c56aa6a4b02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="Rdb26c852b9094ae6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R318a346ccc5b487a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R55c6f2abfea247a4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5516,7 +5516,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="434" t="str">
-        <x:v>Use this checklist after Start is verified. For a manual action, use the small dropdown to select ☑ when complete. Automatic and not-due rows need no action.</x:v>
+        <x:v>Use this checklist after Start is verified. The Codex preview is read-only: tell Codex when a manual action is complete, and this plan will update to Done. Automatic and not-due rows need no action.</x:v>
       </x:c>
       <x:c r="B2" s="434"/>
       <x:c r="C2" s="434"/>
@@ -5571,7 +5571,7 @@
         <x:v>Sep 8–Sep 14 purchases</x:v>
       </x:c>
       <x:c r="C6" s="451" t="str">
-        <x:f>COUNTIFS(F9:F21,"Manual",E9:E21,"☑")&amp;" / "&amp;COUNTIF(F9:F21,"Manual")&amp;" manual payments complete"</x:f>
+        <x:f>COUNTIFS(F9:F21,"Manual",E9:E21,"Done")&amp;" / "&amp;COUNTIF(F9:F21,"Manual")&amp;" manual payments complete"</x:f>
         <x:v>0 / 5 manual payments complete</x:v>
       </x:c>
       <x:c r="D6" s="451" t="str">
@@ -5627,7 +5627,7 @@
         <x:v>786.38</x:v>
       </x:c>
       <x:c r="E9" s="453" t="str">
-        <x:v>☐</x:v>
+        <x:v>Pay today</x:v>
       </x:c>
       <x:c r="F9" s="454" t="str">
         <x:v>Manual</x:v>
@@ -5650,7 +5650,7 @@
         <x:v>106.26</x:v>
       </x:c>
       <x:c r="E10" s="453" t="str">
-        <x:v>☐</x:v>
+        <x:v>Pay today</x:v>
       </x:c>
       <x:c r="F10" s="454" t="str">
         <x:v>Manual</x:v>
@@ -5743,7 +5743,7 @@
         <x:v>148.615</x:v>
       </x:c>
       <x:c r="E14" s="453" t="str">
-        <x:v>☐</x:v>
+        <x:v>Pay today</x:v>
       </x:c>
       <x:c r="F14" s="454" t="str">
         <x:v>Manual</x:v>
@@ -5791,7 +5791,7 @@
         <x:v>172.26230769230767</x:v>
       </x:c>
       <x:c r="E16" s="453" t="str">
-        <x:v>☐</x:v>
+        <x:v>Pay today</x:v>
       </x:c>
       <x:c r="F16" s="454" t="str">
         <x:v>Manual</x:v>
@@ -5907,7 +5907,7 @@
         <x:v>225.157307692308</x:v>
       </x:c>
       <x:c r="E21" s="453" t="str">
-        <x:v>☐</x:v>
+        <x:v>Pay today</x:v>
       </x:c>
       <x:c r="F21" s="454" t="str">
         <x:v>Manual</x:v>
@@ -5998,26 +5998,9 @@
     <x:mergeCell ref="A26:D26"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="E9:E21">
-    <x:cfRule type="containsText" dxfId="23" priority="1" operator="containsText" text="☐"/>
-    <x:cfRule type="containsText" dxfId="24" priority="2" operator="containsText" text="☑"/>
+    <x:cfRule type="containsText" dxfId="23" priority="1" operator="containsText" text="Pay today"/>
+    <x:cfRule type="containsText" dxfId="24" priority="2" operator="containsText" text="Done"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="5">
-    <x:dataValidation type="list" sqref="E9">
-      <x:formula1>"☐,☑"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="E10">
-      <x:formula1>"☐,☑"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="E14">
-      <x:formula1>"☐,☑"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="E16">
-      <x:formula1>"☐,☑"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="E21">
-      <x:formula1>"☐,☑"</x:formula1>
-    </x:dataValidation>
-  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Record Tuesday payments and update funding
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R4f0b57e93c1747d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R875bfa1073d14b5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R8b4037e1d2564583"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R96e6caae1d364830"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R003a1fac39e342a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="Ra5a7789e1a9a4af1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="Rb2a2fa770e0f4dc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R57ee9fe374894332"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="Rc8512f0c80a04a57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R053ab9e7d4b94bf2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R3876ceb680ec423b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R43844c56aa6a4b02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="Rdb26c852b9094ae6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R318a346ccc5b487a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R55c6f2abfea247a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="Rad1cd89545814255"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R9b2a3ac37105439a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R9f729450407f49ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R7f53efa01205468b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="Re7ef60704a114985"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R0b4f727fa3054fae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="Rc3f3f48a8add4b96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="Ra34ac3923c9a486b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="Rd5857b283f9d4d8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R53dc008c9f914066"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="Rd9b417cdbd61429c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="Rc327ac154c534600"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R7f0bd010a9aa49ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="Rcf1ba4797b614d57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="Rdbb734512a814e1e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5572,7 +5572,7 @@
       </x:c>
       <x:c r="C6" s="451" t="str">
         <x:f>COUNTIFS(F9:F21,"Manual",E9:E21,"Done")&amp;" / "&amp;COUNTIF(F9:F21,"Manual")&amp;" manual payments complete"</x:f>
-        <x:v>0 / 5 manual payments complete</x:v>
+        <x:v>4 / 5 manual payments complete</x:v>
       </x:c>
       <x:c r="D6" s="451" t="str">
         <x:v>Current plan — Sep 15</x:v>
@@ -5601,7 +5601,7 @@
         <x:v>Basis</x:v>
       </x:c>
       <x:c r="D8" s="425" t="str">
-        <x:v>Planned amount</x:v>
+        <x:v>Amount</x:v>
       </x:c>
       <x:c r="E8" s="425" t="str">
         <x:v>Status</x:v>
@@ -5621,19 +5621,19 @@
         <x:v>Chase Sapphire</x:v>
       </x:c>
       <x:c r="C9" s="419" t="str">
-        <x:v>Current Sep. 15 balance</x:v>
+        <x:v>Actual Sep. 15 payment</x:v>
       </x:c>
       <x:c r="D9" s="462" t="n">
-        <x:v>786.38</x:v>
+        <x:v>813.84</x:v>
       </x:c>
       <x:c r="E9" s="453" t="str">
-        <x:v>Pay today</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F9" s="454" t="str">
         <x:v>Manual</x:v>
       </x:c>
       <x:c r="G9" s="419" t="str">
-        <x:v>Pay the current balance, including listed pending charges</x:v>
+        <x:v>Paid Sep. 15; actual payment replaces the planned balance</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="28" customHeight="1">
@@ -5644,19 +5644,19 @@
         <x:v>Citi card</x:v>
       </x:c>
       <x:c r="C10" s="419" t="str">
-        <x:v>Current Sep. 15 balance</x:v>
+        <x:v>Actual Sep. 15 payment</x:v>
       </x:c>
       <x:c r="D10" s="462" t="n">
         <x:v>106.26</x:v>
       </x:c>
       <x:c r="E10" s="453" t="str">
-        <x:v>Pay today</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F10" s="454" t="str">
         <x:v>Manual</x:v>
       </x:c>
       <x:c r="G10" s="419" t="str">
-        <x:v>Pay the current balance, including listed pending charges</x:v>
+        <x:v>Paid Sep. 15</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="28" customHeight="1">
@@ -5743,13 +5743,13 @@
         <x:v>148.615</x:v>
       </x:c>
       <x:c r="E14" s="453" t="str">
-        <x:v>Pay today</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F14" s="454" t="str">
         <x:v>Manual</x:v>
       </x:c>
       <x:c r="G14" s="419" t="str">
-        <x:v>Four weekly payments remain before Oct. 10</x:v>
+        <x:v>Paid Sep. 15; preserve the Oct. 10 payoff schedule</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="28" customHeight="1">
@@ -5784,20 +5784,20 @@
         <x:v>Car fund / CUTX</x:v>
       </x:c>
       <x:c r="C16" s="419" t="str">
-        <x:v>Weekly reserve toward Sep. 27 due date</x:v>
+        <x:v>Actual Sep. 15 funding</x:v>
       </x:c>
       <x:c r="D16" s="462" t="n">
         <x:f>'Support - Budget Inputs'!E13</x:f>
         <x:v>172.26230769230767</x:v>
       </x:c>
       <x:c r="E16" s="453" t="str">
-        <x:v>Pay today</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F16" s="454" t="str">
         <x:v>Manual</x:v>
       </x:c>
       <x:c r="G16" s="419" t="str">
-        <x:v>Move to CUTX reserve; do not pay the loan early</x:v>
+        <x:v>Paid Sep. 15</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="28" customHeight="1">
@@ -5904,7 +5904,7 @@
       </x:c>
       <x:c r="D21" s="462" t="n">
         <x:f>MAX(0,E23+E25-E24)</x:f>
-        <x:v>225.157307692308</x:v>
+        <x:v>252.61730769230803</x:v>
       </x:c>
       <x:c r="E21" s="453" t="str">
         <x:v>Pay today</x:v>
@@ -5925,7 +5925,7 @@
       <x:c r="C22" s="451"/>
       <x:c r="D22" s="456" t="n">
         <x:f>SUM(D9:D20)</x:f>
-        <x:v>1616.877307692308</x:v>
+        <x:v>1644.337307692308</x:v>
       </x:c>
       <x:c r="E22" s="419"/>
       <x:c r="F22" s="419"/>
@@ -5940,7 +5940,7 @@
       <x:c r="D23" s="457"/>
       <x:c r="E23" s="463" t="n">
         <x:f>SUM(D9:D20)</x:f>
-        <x:v>1616.877307692308</x:v>
+        <x:v>1644.337307692308</x:v>
       </x:c>
       <x:c r="F23" s="419"/>
       <x:c r="G23" s="419"/>
@@ -5981,7 +5981,7 @@
       <x:c r="D26" s="457"/>
       <x:c r="E26" s="465" t="n">
         <x:f>D21</x:f>
-        <x:v>225.157307692308</x:v>
+        <x:v>252.61730769230803</x:v>
       </x:c>
       <x:c r="F26" s="419"/>
       <x:c r="G26" s="419"/>
@@ -8083,7 +8083,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F7" s="543" t="n">
-        <x:v>1616.8773076923076</x:v>
+        <x:v>1644.337307692308</x:v>
       </x:c>
       <x:c r="G7" s="544" t="str">
         <x:v>Plan created — Sep 15</x:v>
@@ -8105,7 +8105,7 @@
         <x:f>IF(H7="","",H7-K7)</x:f>
       </x:c>
       <x:c r="M7" s="544" t="str">
-        <x:v>Sep. 15 payment plan built from verified imports. It uses a $225.16 general cash top-up from Wealthfront and makes no rent contribution this Tuesday.</x:v>
+        <x:v>Sep. 15 plan updated after the $813.84 Chase payment. It requires a $252.62 general cash top-up from Wealthfront and makes no rent contribution this Tuesday.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Reconcile Chase payment delta
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="Rad1cd89545814255"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R9b2a3ac37105439a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R9f729450407f49ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R7f53efa01205468b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="Re7ef60704a114985"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R0b4f727fa3054fae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="Rc3f3f48a8add4b96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="Ra34ac3923c9a486b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="Rd5857b283f9d4d8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R53dc008c9f914066"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="Rd9b417cdbd61429c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="Rc327ac154c534600"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R7f0bd010a9aa49ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="Rcf1ba4797b614d57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="Rdbb734512a814e1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R8d369dc7c7fe4d18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="Rb4ad9f64c05d4feb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="Ra21610d5f05d469e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R56642d54e1a540be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="Ra388a918106d4c0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R1c20e8e563554a71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="Radb50eb7313a488c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="Rc168b0be4b4a4fec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="Rf60bf00334ed44c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="Ra2320f965b474626"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R45fd8d15d0884546"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R3acf3c66ac7e4956"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R4767f25b9eb743f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R3a2b62663120403d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="Rf7c6dc60ecd942ab"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3143,7 +3143,7 @@
       </x:c>
       <x:c r="B16" s="411" t="n">
         <x:f>COUNTIF('Support - Ledger'!E5:E304,"Pending")</x:f>
-        <x:v>13</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C16" s="403" t="str">
         <x:v>Capture every pending item and keep unclear amounts flagged</x:v>
@@ -3290,7 +3290,7 @@
         <x:v>USD</x:v>
       </x:c>
       <x:c r="G5" s="419" t="str">
-        <x:v>Current balance from Sep. 15 Chase screenshot. No payment is currently due; $159.54 of current activity is pending and tracked separately.</x:v>
+        <x:v>Pre-payment balance from Sep. 15 Chase screenshot. No payment is currently due; the later Sep. 15 capture shows $132.08 of current activity pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -4059,18 +4059,18 @@
         <x:v>Posted ledger rows</x:v>
       </x:c>
       <x:c r="D14" s="419" t="n">
-        <x:v>19</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="E14" s="419" t="n">
         <x:f>COUNTIF('Support - Ledger'!$K$5:$K$304,B14)</x:f>
-        <x:v>19</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="F14" s="474" t="n">
-        <x:v>513.2</x:v>
+        <x:v>540.66</x:v>
       </x:c>
       <x:c r="G14" s="474" t="n">
         <x:f>SUMIF('Support - Ledger'!$K$5:$K$304,B14,'Support - Ledger'!$D$5:$D$304)</x:f>
-        <x:v>513.2</x:v>
+        <x:v>540.66</x:v>
       </x:c>
       <x:c r="H14" s="419" t="str">
         <x:v>Yes</x:v>
@@ -4080,7 +4080,7 @@
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J14" s="419" t="str">
-        <x:v>Posted activity reconciled through Sep. 13</x:v>
+        <x:v>Posted activity and exact payment-delta transition reconciled</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
@@ -4094,18 +4094,18 @@
         <x:v>Pending ledger rows</x:v>
       </x:c>
       <x:c r="D15" s="419" t="n">
-        <x:v>8</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E15" s="419" t="n">
         <x:f>COUNTIF('Support - Ledger'!$K$5:$K$304,B15)</x:f>
-        <x:v>8</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F15" s="474" t="n">
-        <x:v>159.54</x:v>
+        <x:v>132.08</x:v>
       </x:c>
       <x:c r="G15" s="474" t="n">
         <x:f>SUMIF('Support - Ledger'!$K$5:$K$304,B15,'Support - Ledger'!$D$5:$D$304)</x:f>
-        <x:v>159.54</x:v>
+        <x:v>132.08</x:v>
       </x:c>
       <x:c r="H15" s="419" t="str">
         <x:v>Yes</x:v>
@@ -4115,7 +4115,7 @@
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J15" s="419" t="str">
-        <x:v>Eight current pending charges reconciled</x:v>
+        <x:v>Six current pending charges reconciled</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
@@ -6137,11 +6137,11 @@
       </x:c>
       <x:c r="C7" s="474" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$F$5:$F$304,A7,'Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$E$5:$E$304,"Posted",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>0</x:v>
+        <x:v>20.91</x:v>
       </x:c>
       <x:c r="D7" s="474" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$F$5:$F$304,A7,'Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$E$5:$E$304,"Pending",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>20.91</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E7" s="474" t="n">
         <x:f>C7+D7</x:f>
@@ -6166,11 +6166,11 @@
       </x:c>
       <x:c r="C8" s="474" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$F$5:$F$304,A8,'Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$E$5:$E$304,"Posted",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>39.42</x:v>
+        <x:v>45.97</x:v>
       </x:c>
       <x:c r="D8" s="474" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$F$5:$F$304,A8,'Support - Ledger'!$H$5:$H$304,$B$3,'Support - Ledger'!$E$5:$E$304,"Pending",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>19</x:v>
+        <x:v>12.45</x:v>
       </x:c>
       <x:c r="E8" s="474" t="n">
         <x:f>C8+D8</x:f>
@@ -6578,11 +6578,11 @@
       </x:c>
       <x:c r="C23" s="476" t="n">
         <x:f>SUM(C6:C21)</x:f>
-        <x:v>391.34000000000003</x:v>
+        <x:v>418.80000000000007</x:v>
       </x:c>
       <x:c r="D23" s="476" t="n">
         <x:f>SUM(D6:D21)</x:f>
-        <x:v>154.79</x:v>
+        <x:v>127.33000000000001</x:v>
       </x:c>
       <x:c r="E23" s="476" t="n">
         <x:f>SUM(E6:E21)</x:f>
@@ -8091,11 +8091,11 @@
       <x:c r="H7" s="543"/>
       <x:c r="I7" s="474" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$H$5:$H$304,B7,'Support - Ledger'!$E$5:$E$304,"Posted",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>414.81</x:v>
+        <x:v>442.27000000000004</x:v>
       </x:c>
       <x:c r="J7" s="474" t="n">
         <x:f>SUMIFS('Support - Ledger'!$D$5:$D$304,'Support - Ledger'!$H$5:$H$304,B7,'Support - Ledger'!$E$5:$E$304,"Pending",'Support - Ledger'!$G$5:$G$304,"Include",'Support - Ledger'!$M$5:$M$304,"Verified")</x:f>
-        <x:v>154.79</x:v>
+        <x:v>127.33</x:v>
       </x:c>
       <x:c r="K7" s="474" t="n">
         <x:f>I7+J7</x:f>
@@ -12941,7 +12941,7 @@
         <x:v>20.91</x:v>
       </x:c>
       <x:c r="E98" s="544" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Posted</x:v>
       </x:c>
       <x:c r="F98" s="544" t="str">
         <x:v>DoorDash</x:v>
@@ -12957,13 +12957,13 @@
         <x:v>chase-2026-09-13-doordash-2091</x:v>
       </x:c>
       <x:c r="J98" s="544" t="str">
-        <x:v>Pending in Sep. 15 Chase activity</x:v>
+        <x:v>No longer pending in the later Sep. 15 capture; $20.91 is part of the exact $27.46 Chase-payment delta</x:v>
       </x:c>
       <x:c r="K98" s="544" t="str">
-        <x:v>Chase pending — Sep 15</x:v>
+        <x:v>Chase activity — Sep 15</x:v>
       </x:c>
       <x:c r="L98" s="544" t="str">
-        <x:v>Pending list</x:v>
+        <x:v>Posted activity</x:v>
       </x:c>
       <x:c r="M98" s="544" t="str">
         <x:v>Verified</x:v>
@@ -12983,7 +12983,7 @@
         <x:v>6.55</x:v>
       </x:c>
       <x:c r="E99" s="544" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Posted</x:v>
       </x:c>
       <x:c r="F99" s="544" t="str">
         <x:v>Starbucks</x:v>
@@ -12999,13 +12999,13 @@
         <x:v>chase-2026-09-13-starbucks-655</x:v>
       </x:c>
       <x:c r="J99" s="544" t="str">
-        <x:v>Pending in Sep. 15 Chase activity</x:v>
+        <x:v>No longer pending in the later Sep. 15 capture; $6.55 is part of the exact $27.46 Chase-payment delta</x:v>
       </x:c>
       <x:c r="K99" s="544" t="str">
-        <x:v>Chase pending — Sep 15</x:v>
+        <x:v>Chase activity — Sep 15</x:v>
       </x:c>
       <x:c r="L99" s="544" t="str">
-        <x:v>Pending list</x:v>
+        <x:v>Posted activity</x:v>
       </x:c>
       <x:c r="M99" s="544" t="str">
         <x:v>Verified</x:v>

</xml_diff>

<commit_message>
Record Wealthfront transfer completion
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R8d369dc7c7fe4d18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="Rb4ad9f64c05d4feb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="Ra21610d5f05d469e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R56642d54e1a540be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="Ra388a918106d4c0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R1c20e8e563554a71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="Radb50eb7313a488c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="Rc168b0be4b4a4fec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="Rf60bf00334ed44c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="Ra2320f965b474626"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R45fd8d15d0884546"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R3acf3c66ac7e4956"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R4767f25b9eb743f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R3a2b62663120403d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="Rf7c6dc60ecd942ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R0f1a8cc687674025"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="Rb41006b3b9bd438b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R0c6cf017267641a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R6f8fb1f293694fc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R408530568b73488d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="Red5bf85d75c141cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R1a01c765493f4e0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R17e716ec5fbe451b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="Rade7f0c896f54117"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R698a351f760549d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R7aa217eda4594238"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="Rd62a0a7986aa4b95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="Ra39c0884caf24c87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R9529d60e524c45d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R40b48c0ff03942bf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5572,7 +5572,7 @@
       </x:c>
       <x:c r="C6" s="451" t="str">
         <x:f>COUNTIFS(F9:F21,"Manual",E9:E21,"Done")&amp;" / "&amp;COUNTIF(F9:F21,"Manual")&amp;" manual payments complete"</x:f>
-        <x:v>4 / 5 manual payments complete</x:v>
+        <x:v>5 / 5 manual payments complete</x:v>
       </x:c>
       <x:c r="D6" s="451" t="str">
         <x:v>Current plan — Sep 15</x:v>
@@ -5907,14 +5907,13 @@
         <x:v>252.61730769230803</x:v>
       </x:c>
       <x:c r="E21" s="453" t="str">
-        <x:v>Pay today</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F21" s="454" t="str">
         <x:v>Manual</x:v>
       </x:c>
       <x:c r="G21" s="419" t="str">
-        <x:f>IF(D21=0,"No transfer needed; leave $1 in Wells","Transfer this amount from Wealthfront to leave $1 in Wells")</x:f>
-        <x:v>Transfer this amount from Wealthfront to leave $1 in Wells</x:v>
+        <x:v>Transferred Sep. 15; user confirmed</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -8086,7 +8085,7 @@
         <x:v>1644.337307692308</x:v>
       </x:c>
       <x:c r="G7" s="544" t="str">
-        <x:v>Plan created — Sep 15</x:v>
+        <x:v>Manual actions completed — Sep 15</x:v>
       </x:c>
       <x:c r="H7" s="543"/>
       <x:c r="I7" s="474" t="n">
@@ -8105,7 +8104,7 @@
         <x:f>IF(H7="","",H7-K7)</x:f>
       </x:c>
       <x:c r="M7" s="544" t="str">
-        <x:v>Sep. 15 plan updated after the $813.84 Chase payment. It requires a $252.62 general cash top-up from Wealthfront and makes no rent contribution this Tuesday.</x:v>
+        <x:v>All five Sep. 15 manual actions are user-confirmed complete, including the $252.62 Wealthfront top-up. Automatic transfers remain for next-import verification.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="22" customHeight="1">
@@ -8902,7 +8901,7 @@
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="G5:G30">
-      <x:formula1>"In progress,Plan created — Sep 9,Plan created — Sep 15,Data verified — Sep 9,Legacy — not source-audited,✓ Completed,Needs review"</x:formula1>
+      <x:formula1>"In progress,Plan created — Sep 9,Plan created — Sep 15,Manual actions completed — Sep 15,Data verified — Sep 9,Legacy — not source-audited,✓ Completed,Needs review"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Streamline weekly workbook refresh
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R0f1a8cc687674025"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="Rb41006b3b9bd438b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R0c6cf017267641a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R6f8fb1f293694fc9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R408530568b73488d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="Red5bf85d75c141cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R1a01c765493f4e0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R17e716ec5fbe451b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="Rade7f0c896f54117"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R698a351f760549d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R7aa217eda4594238"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="Rd62a0a7986aa4b95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="Ra39c0884caf24c87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R9529d60e524c45d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R40b48c0ff03942bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R04983d04dab14ee3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="Rf2348cc516f94bdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="Rf543e083ac464e80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R6bd79b40dc914804"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R8dc8ccf203ef48f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R75eb82a779fa4d85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R73aca529bb104af8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R952d52cd3a714850"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R24641264240a4b68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R6fe4b8abbf67498e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R99a59519899a44da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R69d137c3d783449b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R3259a45ef04d45da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="Rba9bbc63c45e4ace"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R4718fc3f61b74869"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2842,7 +2842,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="434" t="str">
-        <x:v>Open this page during the import. Wells updates first; the current cash plan is built only after every required source is verified. Use Tuesday Review only after that handoff.</x:v>
+        <x:v>Open this page only during the weekly import. Wells updates first; the cash plan is built only after every required source is verified. During import and payment execution, updates stay limited to Start, Tuesday Review, and the transaction ledger.</x:v>
       </x:c>
       <x:c r="B2" s="434"/>
       <x:c r="C2" s="434"/>
@@ -2933,10 +2933,10 @@
         <x:v>Cash plan</x:v>
       </x:c>
       <x:c r="B7" s="438" t="str">
-        <x:v>Built</x:v>
+        <x:v>Manual actions complete</x:v>
       </x:c>
       <x:c r="C7" s="429" t="str">
-        <x:v>Tuesday Review reflects all verified current actions</x:v>
+        <x:v>Automatic transfers await next import</x:v>
       </x:c>
       <x:c r="D7" s="419"/>
       <x:c r="E7" s="401" t="str">
@@ -2958,10 +2958,10 @@
         <x:v>Next action</x:v>
       </x:c>
       <x:c r="B8" s="439" t="str">
-        <x:v>Execute plan</x:v>
+        <x:v>Verify automatics</x:v>
       </x:c>
       <x:c r="C8" s="432" t="str">
-        <x:v>Use Tuesday Review checkoffs while you pay or transfer funds</x:v>
+        <x:v>At the next weekly import, confirm automatic transfers from account activity</x:v>
       </x:c>
       <x:c r="D8" s="419"/>
       <x:c r="E8" s="401" t="str">
@@ -3275,7 +3275,7 @@
         <x:v>Chase card</x:v>
       </x:c>
       <x:c r="B5" s="543" t="n">
-        <x:v>786.38</x:v>
+        <x:v>132.08</x:v>
       </x:c>
       <x:c r="C5" s="543" t="n">
         <x:v>0</x:v>
@@ -3290,7 +3290,7 @@
         <x:v>USD</x:v>
       </x:c>
       <x:c r="G5" s="419" t="str">
-        <x:v>Pre-payment balance from Sep. 15 Chase screenshot. No payment is currently due; the later Sep. 15 capture shows $132.08 of current activity pending.</x:v>
+        <x:v>Current post-payment exposure. The $813.84 payment cleared the $786.38 pre-payment balance plus the $27.46 that posted; six pending charges total $132.08.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -5436,13 +5436,13 @@
         <x:v>Card balance, spending, subscriptions</x:v>
       </x:c>
       <x:c r="C11" s="419" t="str">
-        <x:v>Jun-Aug 2026</x:v>
+        <x:v>Jun-Aug 2026 and Sep. 15 follow-up</x:v>
       </x:c>
       <x:c r="D11" s="419" t="str">
         <x:v>Invincibles app charges: $596.43, $605.63, then $972.68 across the three statement periods; Spectrum internet, Max, dog grooming, and BudgetPetCare observed</x:v>
       </x:c>
       <x:c r="E11" s="419" t="str">
-        <x:v>BudgetPetCare last charged $36.45 on Jul. 29 and recurs every 3 months (next Oct. 16). Spectrum Mobile $672.29 was a one-time phone payoff funded from Wealthfront. Game/app budget cap set to $50/week. SiriusXM, NordVPN, HWBTPLUS, and Max are cancelled and excluded.</x:v>
+        <x:v>Sep. 15 follow-up: six pending charges total $132.08. DoorDash $20.91 and Starbucks $6.55 posted, matching the $27.46 Chase payment difference. BudgetPetCare last charged $36.45 on Jul. 29 and recurs every 3 months (next Oct. 16). Spectrum Mobile $672.29 was a one-time phone payoff funded from Wealthfront. Game/app budget cap set to $50/week. SiriusXM, NordVPN, HWBTPLUS, and Max are cancelled and excluded.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -6033,7 +6033,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="434" t="str">
-        <x:v>Review new purchases against their weekly category limits here. Pending charges count so the week cannot look safer than it is. This is analysis, not the cash decision for today; payments and transfers do not belong here. Only source-verified ledger rows are counted.</x:v>
+        <x:v>Closeout analysis for new purchases against weekly category limits. Pending charges count so the week cannot look safer than it is. This is not the cash decision for today; payments and transfers do not belong here. Only source-verified ledger rows are counted.</x:v>
       </x:c>
       <x:c r="B2" s="434"/>
       <x:c r="C2" s="434"/>
@@ -6667,7 +6667,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="434" t="str">
-        <x:v>Use this ongoing guide after the live Tuesday Review. It reflects the Sep. 9 import inputs; the current rent contribution is calculated in Tuesday Review and recorded in Savings &amp; Debt.</x:v>
+        <x:v>This guide refreshes at weekly closeout. During the import and Tuesday payment execution, use Start and Tuesday Review only. Savings &amp; Debt records the current rent contribution.</x:v>
       </x:c>
       <x:c r="B2" s="434"/>
       <x:c r="C2" s="434"/>

</xml_diff>

<commit_message>
Preserve additive safe cash and confirmed savings
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R04983d04dab14ee3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="Rf2348cc516f94bdd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="Rf543e083ac464e80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R6bd79b40dc914804"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R8dc8ccf203ef48f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R75eb82a779fa4d85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R73aca529bb104af8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R952d52cd3a714850"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R24641264240a4b68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R6fe4b8abbf67498e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R99a59519899a44da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R69d137c3d783449b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R3259a45ef04d45da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="Rba9bbc63c45e4ace"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R4718fc3f61b74869"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R2a974f4e95454df4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="Rb72f53deb76f4e9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R3587b109c3b94d00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R5e2a651303eb4895"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R30d9b4cf779e44da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R77b498eb99c54980"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="Re62cdb7bc5bb4d48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="Rc4188cba3c934cbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R4c44810e9af64359"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R2e643984549a44a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="Rbadd843268084653"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R42c3f5c7ca1d4ff0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R3e108b8a13f148c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R0ff996d7c0ae477f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R570abb20b963491d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3903,7 +3903,7 @@
         <x:v>Personal safe cash</x:v>
       </x:c>
       <x:c r="C7" s="474" t="n">
-        <x:v>510</x:v>
+        <x:v>730</x:v>
       </x:c>
       <x:c r="D7" s="474" t="n">
         <x:v>0</x:v>
@@ -3912,10 +3912,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F7" s="474" t="n">
-        <x:v>510</x:v>
+        <x:v>730</x:v>
       </x:c>
       <x:c r="G7" s="419" t="str">
-        <x:v>Current user-reported personal-safe cash balance. Savings-only and excluded from Wells/Wealthfront funding and spending-capacity calculations.</x:v>
+        <x:v>Additive balance: $220 prior safe cash + $510 Sep. 15 addition = $730. Savings-only and excluded from Wells/Wealthfront funding and spending-capacity calculations.</x:v>
       </x:c>
       <x:c r="H7" s="569"/>
       <x:c r="I7" s="569"/>
@@ -5326,10 +5326,10 @@
         <x:v>Sep 9, 2026</x:v>
       </x:c>
       <x:c r="D4" s="419" t="str">
-        <x:v>Available Wells $1,227.78 after pending Fidelity debit; personal-safe balance $220 includes the earlier $60 plus an additional $160</x:v>
+        <x:v>Available Wells $1,227.78 after pending Fidelity debit; personal-safe balance was $220 after the earlier $60 and additional $160</x:v>
       </x:c>
       <x:c r="E4" s="419" t="str">
-        <x:v>The earlier Jul–Aug account history establishes the $1,343.37 recurring-payroll baseline and $75 weekly Fidelity transfer. Personal-safe cash is savings-only and excluded from Wells cash-plan and spending-capacity calculations. The Sep. 9 Wells balance controls this live review.</x:v>
+        <x:v>The earlier Jul–Aug account history establishes the $1,343.37 recurring-payroll baseline and $75 weekly Fidelity transfer. Personal-safe cash is savings-only and excluded from Wells cash-plan and spending-capacity calculations. On Sep. 15, an additional $510 brought personal-safe cash to $730.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -7045,7 +7045,7 @@
       </x:c>
       <x:c r="B26" s="504" t="n">
         <x:f>'Support - Account Snapshots'!F7</x:f>
-        <x:v>510</x:v>
+        <x:v>730</x:v>
       </x:c>
       <x:c r="C26" s="460"/>
       <x:c r="D26" s="460"/>
@@ -7304,7 +7304,7 @@
       </x:c>
       <x:c r="B6" s="559" t="n">
         <x:f>'Support - Account Snapshots'!F7</x:f>
-        <x:v>510</x:v>
+        <x:v>730</x:v>
       </x:c>
       <x:c r="C6" s="536" t="str">
         <x:v>Rent due estimate</x:v>
@@ -7322,7 +7322,7 @@
       </x:c>
       <x:c r="B7" s="560" t="n">
         <x:f>SUM(B5:B6)</x:f>
-        <x:v>12536.13</x:v>
+        <x:v>12756.13</x:v>
       </x:c>
       <x:c r="C7" s="536" t="str">
         <x:v>Tagged rent reserve</x:v>
@@ -7358,7 +7358,7 @@
       </x:c>
       <x:c r="B9" s="562" t="n">
         <x:f>B7-B8</x:f>
-        <x:v>550.1722999999965</x:v>
+        <x:v>770.1722999999965</x:v>
       </x:c>
       <x:c r="C9" s="541" t="str">
         <x:v>Confirmed funding vs. monthly plan</x:v>
@@ -7412,11 +7412,11 @@
         <x:v>75</x:v>
       </x:c>
       <x:c r="C13" s="544" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D13" s="474" t="n">
         <x:f>B13*C13</x:f>
-        <x:v>0</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="E13" s="419"/>
       <x:c r="F13" s="419"/>
@@ -7429,11 +7429,11 @@
         <x:v>85</x:v>
       </x:c>
       <x:c r="C14" s="544" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D14" s="474" t="n">
         <x:f>B14*C14</x:f>
-        <x:v>0</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="E14" s="419"/>
       <x:c r="F14" s="419"/>
@@ -7446,11 +7446,11 @@
         <x:v>193.36</x:v>
       </x:c>
       <x:c r="C15" s="544" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D15" s="474" t="n">
         <x:f>B15*C15</x:f>
-        <x:v>0</x:v>
+        <x:v>193.36</x:v>
       </x:c>
       <x:c r="E15" s="419"/>
       <x:c r="F15" s="419"/>
@@ -7463,11 +7463,11 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="C16" s="544" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D16" s="474" t="n">
         <x:f>B16*C16</x:f>
-        <x:v>0</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="E16" s="419"/>
       <x:c r="F16" s="419"/>
@@ -7483,7 +7483,7 @@
       <x:c r="C17" s="546"/>
       <x:c r="D17" s="546" t="n">
         <x:f>SUM(D13:D16)</x:f>
-        <x:v>0</x:v>
+        <x:v>403.36</x:v>
       </x:c>
       <x:c r="E17" s="419"/>
       <x:c r="F17" s="419"/>
@@ -16764,7 +16764,7 @@
       </x:c>
       <x:c r="C7" s="452" t="n">
         <x:f>'Support - Account Snapshots'!F7</x:f>
-        <x:v>510</x:v>
+        <x:v>730</x:v>
       </x:c>
       <x:c r="D7" s="452" t="n">
         <x:v>0</x:v>

</xml_diff>

<commit_message>
Enforce batch weekly import workflow
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R2a974f4e95454df4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="Rb72f53deb76f4e9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R3587b109c3b94d00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R5e2a651303eb4895"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R30d9b4cf779e44da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R77b498eb99c54980"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="Re62cdb7bc5bb4d48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="Rc4188cba3c934cbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R4c44810e9af64359"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R2e643984549a44a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="Rbadd843268084653"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R42c3f5c7ca1d4ff0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R3e108b8a13f148c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R0ff996d7c0ae477f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R570abb20b963491d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R7eda423ba42b4f88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R57408b45550d4af5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R658cf2fd3ed64f2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="Raf2546b7c33a4002"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="Rd7e3e67ee6b6482d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R9a9c84de7d11449a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R00c5e8c35b014b01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R55a2cc21586a46c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R795e2d05ce5e4418"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R6efc7324b8a743c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="Re9de26b735cb460c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="Rad45eb4845774d1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="Rd571b5f6c42144d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="Rf541b46bfd03489f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R0d15309ee99e4883"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Add lightweight weekly budget workflow
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R411c0d39414b472b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R60103968d5444b54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R4177a1613d154609"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R84568a1753574085"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R9c100a4440e64a0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R1903a3a9d0d0459a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R54f1b9d1d5fc4e6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R908c7be0a2b6463c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R971532902c814c87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="Re0616269ad994d24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R79d266b62fdb4509"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="Rf9c6ac62416f4321"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R0df290b54da84f72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="Rc0d2cadaa0384509"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R93c5141492454b81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R239940f8548e4bc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R3b90b81547a44822"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R0e9a4c30186b4379"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R7b332a3d215545c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="Rd6499533f7834d9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R528666988e76415b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R24ab7261d31e47fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R164bd2dc979a4d57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R65c4ec1535034dd1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="Raf168c43becd46f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R62771f8fca9c408e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R63e928391aaa4207"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R935b10661b734e51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="Rabc0883cfd3249d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R07810481dd104971"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Update AT&T funding detail to confirmed bill
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="Rb27996489b894238"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R90c0604e581343b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R4e5728f33a404aa0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="Rd88105efb02f4cbb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R1684bff0eac64758"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R4f27a47bd431413f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R39682284210c4496"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R29af88dc81964e08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R52e5f5f09e69496f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="Rd95cc0f1396d4275"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R121635175d384b72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R714e283061cb4133"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R8ef5600459544740"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="Re1d0f0a88c71448f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R563cac3ace7c4596"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="Rf4095757a5eb4e36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="Rb27fe889c64d4fb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R5c1eeea2e0a64f0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="Rbad2ad647cbf4f39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R82c29366fd604889"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R842685c4a80d4907"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="Reded2dabfa2c4745"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="Rb7592730ec094426"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R5e25301ae5ac4781"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R55fe9c42ffd04954"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="Rca85fb1ffdaa425e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R099abb609dda4352"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="Rdc45dde908034f39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R4e31bb3c06de41a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R5368f6dd7c644810"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20716,10 +20716,10 @@
         <x:v>Wealthfront to Wells; Wells AutoPay</x:v>
       </x:c>
       <x:c r="G8" s="1098" t="str">
-        <x:v>Reserve this cycle's $88.59</x:v>
+        <x:v>Reserve this cycle's $48.59</x:v>
       </x:c>
       <x:c r="H8" s="1098" t="str">
-        <x:v>Normal baseline remains $65/month; this cycle includes roaming</x:v>
+        <x:v>Confirmed AT&amp;T payment for this cycle is $48.59; normal baseline remains $65/month</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="40" customHeight="1">

</xml_diff>

<commit_message>
Regenerate workbook after main sync
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="Rf4095757a5eb4e36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="Rb27fe889c64d4fb1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R5c1eeea2e0a64f0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="Rbad2ad647cbf4f39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R82c29366fd604889"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R842685c4a80d4907"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="Reded2dabfa2c4745"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="Rb7592730ec094426"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R5e25301ae5ac4781"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R55fe9c42ffd04954"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="Rca85fb1ffdaa425e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R099abb609dda4352"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="Rdc45dde908034f39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R4e31bb3c06de41a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R5368f6dd7c644810"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R7e682f52b7c94bc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R3c895cd2657a4486"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R098a71c07b7d476b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R4087fdb7057c4c1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R27b2762634ad4ec9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R96ddf800feb14bf8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R69dfd91d1eb24f09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="Rf58b3e17f9084f1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R7c5a61756ba64d13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="Rec33250616354b5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R0a25149ca9f04280"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="Ra3eb44e498464a81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R0a64d8c877a34ed8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R7dadca0890374aa1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R825c547bb64b42dd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -6966,10 +6966,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F6" s="1219" t="n">
-        <x:v>12026.13</x:v>
+        <x:v>11773.512692307691</x:v>
       </x:c>
       <x:c r="G6" s="1098" t="str">
-        <x:v>Sep. 15 balance and activity captured; latest visible activity is the Sep. 14 $300 Wells Fargo IFI transfer.</x:v>
+        <x:v>Screenshot balance was $12,026.13. Less the user-confirmed $252.62 transfer to Wells after capture, working Wealthfront balance is $11,773.51.</x:v>
       </x:c>
       <x:c r="H6" s="671"/>
       <x:c r="I6" s="671"/>
@@ -10430,7 +10430,7 @@
       </x:c>
       <x:c r="B5" s="1160" t="n">
         <x:f>'Support - Account Snapshots'!F6</x:f>
-        <x:v>12026.13</x:v>
+        <x:v>11773.512692307691</x:v>
       </x:c>
       <x:c r="C5" s="1154" t="str">
         <x:v>Next rent due</x:v>
@@ -10466,7 +10466,7 @@
       </x:c>
       <x:c r="B7" s="1160" t="n">
         <x:f>SUM(B5:B6)</x:f>
-        <x:v>12756.13</x:v>
+        <x:v>12503.512692307691</x:v>
       </x:c>
       <x:c r="C7" s="1152" t="str">
         <x:v>Tagged rent reserve</x:v>
@@ -10502,7 +10502,7 @@
       </x:c>
       <x:c r="B9" s="1160" t="n">
         <x:f>B7-B8</x:f>
-        <x:v>770.1722999999965</x:v>
+        <x:v>517.5549923076887</x:v>
       </x:c>
       <x:c r="C9" s="1152" t="str">
         <x:v>Confirmed funding vs. monthly plan</x:v>

</xml_diff>

<commit_message>
Reconcile AT&T Wells top-up
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R7e682f52b7c94bc5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R3c895cd2657a4486"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R098a71c07b7d476b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R4087fdb7057c4c1a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R27b2762634ad4ec9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R96ddf800feb14bf8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R69dfd91d1eb24f09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="Rf58b3e17f9084f1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R7c5a61756ba64d13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="Rec33250616354b5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R0a25149ca9f04280"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="Ra3eb44e498464a81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R0a64d8c877a34ed8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R7dadca0890374aa1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R825c547bb64b42dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="Rf6ecfd10b850477d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R7b8b127adc2e4fbc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R8fcd9e73cc3e4507"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R4c24bbc7d987499e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R0da8efcef7e74fe2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R4a157d854e72433b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="Rce00c59959354a29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="Rd7ae3c7a2f454de3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="Rf6ec6728236c451f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="Rb314b6623ed94fe5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="Ra8020f4f525e4f0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R1e8f838dc1af4e9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R5a3508db04294437"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R1e3f508581424ad8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R72137bad6a9d4284"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -6966,10 +6966,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F6" s="1219" t="n">
-        <x:v>11773.512692307691</x:v>
+        <x:v>11724.922692307691</x:v>
       </x:c>
       <x:c r="G6" s="1098" t="str">
-        <x:v>Screenshot balance was $12,026.13. Less the user-confirmed $252.62 transfer to Wells after capture, working Wealthfront balance is $11,773.51.</x:v>
+        <x:v>Screenshot balance was $12,026.13. Less the user-confirmed $301.21 total transfer to Wells after capture ($252.62 initially plus $48.59 AT&amp;T top-up), working Wealthfront balance is $11,724.92.</x:v>
       </x:c>
       <x:c r="H6" s="671"/>
       <x:c r="I6" s="671"/>
@@ -8672,7 +8672,7 @@
       </x:c>
       <x:c r="C6" s="991" t="str">
         <x:f>COUNTIFS(F9:F22,"Manual",E9:E22,"Done")&amp;" / "&amp;COUNTIF(F9:F22,"Manual")&amp;" manual payments complete</x:f>
-        <x:v>4 / 5 manual payments complete</x:v>
+        <x:v>5 / 5 manual payments complete</x:v>
       </x:c>
       <x:c r="D6" s="991" t="str">
         <x:v>Current plan — Sep 15</x:v>
@@ -9030,13 +9030,13 @@
         <x:v>301.20730769230795</x:v>
       </x:c>
       <x:c r="E22" s="1045" t="str">
-        <x:v>Needs review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F22" s="1046" t="str">
         <x:v>Manual</x:v>
       </x:c>
       <x:c r="G22" s="1047" t="str">
-        <x:v>Actual Sep. 15 top-up was $252.62; the corrected plan includes AT&amp;T before protecting the Wells minimum</x:v>
+        <x:v>Completed: $252.62 initial transfer plus $48.59 AT&amp;T top-up, for a $301.21 total transfer.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="29" customHeight="1">
@@ -10430,7 +10430,7 @@
       </x:c>
       <x:c r="B5" s="1160" t="n">
         <x:f>'Support - Account Snapshots'!F6</x:f>
-        <x:v>11773.512692307691</x:v>
+        <x:v>11724.922692307691</x:v>
       </x:c>
       <x:c r="C5" s="1154" t="str">
         <x:v>Next rent due</x:v>
@@ -10466,7 +10466,7 @@
       </x:c>
       <x:c r="B7" s="1160" t="n">
         <x:f>SUM(B5:B6)</x:f>
-        <x:v>12503.512692307691</x:v>
+        <x:v>12454.922692307691</x:v>
       </x:c>
       <x:c r="C7" s="1152" t="str">
         <x:v>Tagged rent reserve</x:v>
@@ -10502,7 +10502,7 @@
       </x:c>
       <x:c r="B9" s="1160" t="n">
         <x:f>B7-B8</x:f>
-        <x:v>517.5549923076887</x:v>
+        <x:v>468.9649923076886</x:v>
       </x:c>
       <x:c r="C9" s="1152" t="str">
         <x:v>Confirmed funding vs. monthly plan</x:v>
@@ -11233,10 +11233,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F7" s="1166" t="n">
-        <x:v>1644.337307692308</x:v>
+        <x:v>1692.927307692308</x:v>
       </x:c>
       <x:c r="G7" s="1167" t="str">
-        <x:v>Needs review</x:v>
+        <x:v>Manual actions completed — Sep 15</x:v>
       </x:c>
       <x:c r="H7" s="1166"/>
       <x:c r="I7" s="1168" t="n">
@@ -11255,7 +11255,7 @@
         <x:f>IF(H7="","",H7-K7)</x:f>
       </x:c>
       <x:c r="M7" s="1167" t="str">
-        <x:v>The Sep. 15 plan omitted the user-confirmed $48.59 AT&amp;T Wells payment. The original plan amount remains preserved; reconcile the resulting Wells shortfall before treating this week as complete.</x:v>
+        <x:v>All five Sep. 15 manual actions are user-confirmed complete. The Wealthfront top-up totals $301.21: $252.62 initially plus the $48.59 AT&amp;T top-up. Automatic transfers remain for next-import verification.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="26" customHeight="1">

</xml_diff>